<commit_message>
Ficha de terreno: hasta 14 actividades; fondos con alarife (líquido tras retención 15,25%) y arriendo de caballos (+IVA 19%); plantilla ampliada; SW v14. Verificado con datos de prueba.
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/plantilla_ficha_terreno.xlsx
+++ b/assets/plantilla_ficha_terreno.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informe PLANIFICACION" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Informe PLANIFICACION'!$B$1:$P$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Informe PLANIFICACION'!$B$1:$P$71</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2356,7 +2356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T86"/>
+  <dimension ref="A1:T94"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="68.7109375" customWidth="1" min="2" max="2"/>
@@ -3856,209 +3856,209 @@
       <c r="O40" s="275" t="n"/>
       <c r="P40" s="270" t="n"/>
     </row>
-    <row r="41" ht="21.75" customHeight="1" thickBot="1">
+    <row r="41" ht="18.75" customHeight="1" thickBot="1">
       <c r="B41" s="291" t="n"/>
-      <c r="C41" s="187" t="inlineStr">
+      <c r="C41" s="153" t="inlineStr">
+        <is>
+          <t>Alarife (líquido)</t>
+        </is>
+      </c>
+      <c r="D41" s="270" t="n"/>
+      <c r="E41" s="280" t="inlineStr">
+        <is>
+          <t>@@FONDOS_ALARIFE@@</t>
+        </is>
+      </c>
+      <c r="F41" s="270" t="n"/>
+      <c r="G41" s="227" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_ALARIFE@@</t>
+        </is>
+      </c>
+      <c r="H41" s="275" t="n"/>
+      <c r="I41" s="275" t="n"/>
+      <c r="J41" s="275" t="n"/>
+      <c r="K41" s="275" t="n"/>
+      <c r="L41" s="275" t="n"/>
+      <c r="M41" s="275" t="n"/>
+      <c r="N41" s="275" t="n"/>
+      <c r="O41" s="275" t="n"/>
+      <c r="P41" s="270" t="n"/>
+    </row>
+    <row r="42" ht="18.75" customHeight="1" thickBot="1">
+      <c r="B42" s="291" t="n"/>
+      <c r="C42" s="153" t="inlineStr">
+        <is>
+          <t>Arriendo de caballos (c/ IVA)</t>
+        </is>
+      </c>
+      <c r="D42" s="270" t="n"/>
+      <c r="E42" s="280" t="inlineStr">
+        <is>
+          <t>@@FONDOS_CABALLOS@@</t>
+        </is>
+      </c>
+      <c r="F42" s="270" t="n"/>
+      <c r="G42" s="227" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_CABALLOS@@</t>
+        </is>
+      </c>
+      <c r="H42" s="275" t="n"/>
+      <c r="I42" s="275" t="n"/>
+      <c r="J42" s="275" t="n"/>
+      <c r="K42" s="275" t="n"/>
+      <c r="L42" s="275" t="n"/>
+      <c r="M42" s="275" t="n"/>
+      <c r="N42" s="275" t="n"/>
+      <c r="O42" s="275" t="n"/>
+      <c r="P42" s="270" t="n"/>
+    </row>
+    <row r="43" ht="21.75" customHeight="1" thickBot="1">
+      <c r="B43" s="291" t="n"/>
+      <c r="C43" s="187" t="inlineStr">
         <is>
           <t>@@FONDOS_OTRO_LABEL@@</t>
         </is>
       </c>
-      <c r="D41" s="271" t="n"/>
-      <c r="E41" s="280" t="inlineStr">
+      <c r="D43" s="271" t="n"/>
+      <c r="E43" s="280" t="inlineStr">
         <is>
           <t>@@FONDOS_E41@@</t>
         </is>
       </c>
-      <c r="F41" s="270" t="n"/>
-      <c r="G41" s="231" t="inlineStr">
+      <c r="F43" s="270" t="n"/>
+      <c r="G43" s="231" t="inlineStr">
         <is>
           <t>@@FONDOS_DET_G41@@</t>
         </is>
       </c>
-      <c r="H41" s="276" t="n"/>
-      <c r="I41" s="276" t="n"/>
-      <c r="J41" s="276" t="n"/>
-      <c r="K41" s="276" t="n"/>
-      <c r="L41" s="276" t="n"/>
-      <c r="M41" s="276" t="n"/>
-      <c r="N41" s="276" t="n"/>
-      <c r="O41" s="276" t="n"/>
-      <c r="P41" s="271" t="n"/>
-    </row>
-    <row r="42" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B42" s="294" t="n"/>
-      <c r="C42" s="200" t="inlineStr">
+      <c r="H43" s="276" t="n"/>
+      <c r="I43" s="276" t="n"/>
+      <c r="J43" s="276" t="n"/>
+      <c r="K43" s="276" t="n"/>
+      <c r="L43" s="276" t="n"/>
+      <c r="M43" s="276" t="n"/>
+      <c r="N43" s="276" t="n"/>
+      <c r="O43" s="276" t="n"/>
+      <c r="P43" s="271" t="n"/>
+    </row>
+    <row r="44" ht="22.5" customHeight="1" thickBot="1">
+      <c r="B44" s="294" t="n"/>
+      <c r="C44" s="200" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D42" s="295" t="n"/>
-      <c r="E42" s="296" t="inlineStr">
+      <c r="D44" s="295" t="n"/>
+      <c r="E44" s="296" t="inlineStr">
         <is>
           <t>@@FONDOS_E42@@</t>
         </is>
       </c>
-      <c r="F42" s="253" t="n"/>
-      <c r="G42" s="197" t="n"/>
-      <c r="Q42" s="13" t="n"/>
-      <c r="R42" s="13" t="n"/>
-    </row>
-    <row r="43" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B43" s="7" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="197" t="n"/>
-      <c r="F43" s="197" t="n"/>
-      <c r="G43" s="197" t="n"/>
-      <c r="H43" s="197" t="n"/>
-      <c r="I43" s="197" t="n"/>
-      <c r="J43" s="197" t="n"/>
-      <c r="K43" s="197" t="n"/>
-      <c r="L43" s="197" t="n"/>
-      <c r="M43" s="197" t="n"/>
-      <c r="N43" s="197" t="n"/>
-      <c r="Q43" s="13" t="n"/>
-      <c r="R43" s="13" t="n"/>
-    </row>
-    <row r="44" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B44" s="104" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES / OBJETIVOS</t>
-        </is>
-      </c>
-      <c r="C44" s="229" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="D44" s="106" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> # DIAS</t>
-        </is>
-      </c>
-      <c r="E44" s="229" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD / OBJETIVO</t>
-        </is>
-      </c>
-      <c r="F44" s="84" t="n"/>
-      <c r="G44" s="84" t="n"/>
-      <c r="H44" s="84" t="n"/>
-      <c r="I44" s="84" t="n"/>
-      <c r="J44" s="84" t="n"/>
-      <c r="K44" s="84" t="n"/>
-      <c r="L44" s="84" t="n"/>
-      <c r="M44" s="84" t="n"/>
-      <c r="N44" s="84" t="n"/>
-      <c r="O44" s="84" t="n"/>
-      <c r="P44" s="268" t="n"/>
+      <c r="F44" s="253" t="n"/>
+      <c r="G44" s="197" t="n"/>
       <c r="Q44" s="13" t="n"/>
       <c r="R44" s="13" t="n"/>
     </row>
     <row r="45" ht="22.5" customHeight="1">
-      <c r="B45" s="181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detalle de actividades (diarias o por periodos) u objetivos a realizar durante cometido </t>
-        </is>
-      </c>
-      <c r="C45" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="103" t="inlineStr">
-        <is>
-          <t>@@ACT1_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E45" s="235" t="inlineStr">
-        <is>
-          <t>@@ACT1_DESC@@</t>
-        </is>
-      </c>
-      <c r="F45" s="257" t="n"/>
-      <c r="G45" s="257" t="n"/>
-      <c r="H45" s="257" t="n"/>
-      <c r="I45" s="257" t="n"/>
-      <c r="J45" s="257" t="n"/>
-      <c r="K45" s="257" t="n"/>
-      <c r="L45" s="257" t="n"/>
-      <c r="M45" s="257" t="n"/>
-      <c r="N45" s="257" t="n"/>
-      <c r="O45" s="257" t="n"/>
-      <c r="P45" s="258" t="n"/>
+      <c r="B45" s="7" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+      <c r="E45" s="197" t="n"/>
+      <c r="F45" s="197" t="n"/>
+      <c r="G45" s="197" t="n"/>
+      <c r="H45" s="197" t="n"/>
+      <c r="I45" s="197" t="n"/>
+      <c r="J45" s="197" t="n"/>
+      <c r="K45" s="197" t="n"/>
+      <c r="L45" s="197" t="n"/>
+      <c r="M45" s="197" t="n"/>
+      <c r="N45" s="197" t="n"/>
       <c r="Q45" s="13" t="n"/>
       <c r="R45" s="13" t="n"/>
     </row>
     <row r="46" ht="22.5" customHeight="1">
-      <c r="B46" s="297" t="n"/>
-      <c r="C46" s="141" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" s="21" t="inlineStr">
-        <is>
-          <t>@@ACT2_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E46" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT2_DESC@@</t>
-        </is>
-      </c>
-      <c r="F46" s="275" t="n"/>
-      <c r="G46" s="275" t="n"/>
-      <c r="H46" s="275" t="n"/>
-      <c r="I46" s="275" t="n"/>
-      <c r="J46" s="275" t="n"/>
-      <c r="K46" s="275" t="n"/>
-      <c r="L46" s="275" t="n"/>
-      <c r="M46" s="275" t="n"/>
-      <c r="N46" s="275" t="n"/>
-      <c r="O46" s="275" t="n"/>
-      <c r="P46" s="270" t="n"/>
+      <c r="B46" s="104" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES / OBJETIVOS</t>
+        </is>
+      </c>
+      <c r="C46" s="229" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D46" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> # DIAS</t>
+        </is>
+      </c>
+      <c r="E46" s="229" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD / OBJETIVO</t>
+        </is>
+      </c>
+      <c r="F46" s="84" t="n"/>
+      <c r="G46" s="84" t="n"/>
+      <c r="H46" s="84" t="n"/>
+      <c r="I46" s="84" t="n"/>
+      <c r="J46" s="84" t="n"/>
+      <c r="K46" s="84" t="n"/>
+      <c r="L46" s="84" t="n"/>
+      <c r="M46" s="84" t="n"/>
+      <c r="N46" s="84" t="n"/>
+      <c r="O46" s="84" t="n"/>
+      <c r="P46" s="268" t="n"/>
       <c r="Q46" s="13" t="n"/>
       <c r="R46" s="13" t="n"/>
     </row>
     <row r="47" ht="22.5" customHeight="1">
-      <c r="B47" s="297" t="n"/>
-      <c r="C47" s="141" t="n">
-        <v>3</v>
-      </c>
-      <c r="D47" s="21" t="inlineStr">
-        <is>
-          <t>@@ACT3_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E47" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT3_DESC@@</t>
-        </is>
-      </c>
-      <c r="F47" s="275" t="n"/>
-      <c r="G47" s="275" t="n"/>
-      <c r="H47" s="275" t="n"/>
-      <c r="I47" s="275" t="n"/>
-      <c r="J47" s="275" t="n"/>
-      <c r="K47" s="275" t="n"/>
-      <c r="L47" s="275" t="n"/>
-      <c r="M47" s="275" t="n"/>
-      <c r="N47" s="275" t="n"/>
-      <c r="O47" s="275" t="n"/>
-      <c r="P47" s="270" t="n"/>
+      <c r="B47" s="181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de actividades (diarias o por periodos) u objetivos a realizar durante cometido </t>
+        </is>
+      </c>
+      <c r="C47" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="103" t="inlineStr">
+        <is>
+          <t>@@ACT1_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E47" s="235" t="inlineStr">
+        <is>
+          <t>@@ACT1_DESC@@</t>
+        </is>
+      </c>
+      <c r="F47" s="257" t="n"/>
+      <c r="G47" s="257" t="n"/>
+      <c r="H47" s="257" t="n"/>
+      <c r="I47" s="257" t="n"/>
+      <c r="J47" s="257" t="n"/>
+      <c r="K47" s="257" t="n"/>
+      <c r="L47" s="257" t="n"/>
+      <c r="M47" s="257" t="n"/>
+      <c r="N47" s="257" t="n"/>
+      <c r="O47" s="257" t="n"/>
+      <c r="P47" s="258" t="n"/>
       <c r="Q47" s="13" t="n"/>
       <c r="R47" s="13" t="n"/>
     </row>
     <row r="48" ht="22.5" customHeight="1">
       <c r="B48" s="297" t="n"/>
       <c r="C48" s="141" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
-          <t>@@ACT4_DIAS@@</t>
+          <t>@@ACT2_DIAS@@</t>
         </is>
       </c>
       <c r="E48" s="151" t="inlineStr">
         <is>
-          <t>@@ACT4_DESC@@</t>
+          <t>@@ACT2_DESC@@</t>
         </is>
       </c>
       <c r="F48" s="275" t="n"/>
@@ -4078,16 +4078,16 @@
     <row r="49" ht="22.5" customHeight="1">
       <c r="B49" s="297" t="n"/>
       <c r="C49" s="141" t="n">
-        <v>5</v>
-      </c>
-      <c r="D49" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT5_DIAS@@</t>
+        <v>3</v>
+      </c>
+      <c r="D49" s="21" t="inlineStr">
+        <is>
+          <t>@@ACT3_DIAS@@</t>
         </is>
       </c>
       <c r="E49" s="151" t="inlineStr">
         <is>
-          <t>@@ACT5_DESC@@</t>
+          <t>@@ACT3_DESC@@</t>
         </is>
       </c>
       <c r="F49" s="275" t="n"/>
@@ -4104,19 +4104,19 @@
       <c r="Q49" s="13" t="n"/>
       <c r="R49" s="13" t="n"/>
     </row>
-    <row r="50" ht="18.75" customHeight="1">
+    <row r="50" ht="22.5" customHeight="1">
       <c r="B50" s="297" t="n"/>
       <c r="C50" s="141" t="n">
-        <v>6</v>
-      </c>
-      <c r="D50" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT6_DIAS@@</t>
+        <v>4</v>
+      </c>
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>@@ACT4_DIAS@@</t>
         </is>
       </c>
       <c r="E50" s="151" t="inlineStr">
         <is>
-          <t>@@ACT6_DESC@@</t>
+          <t>@@ACT4_DESC@@</t>
         </is>
       </c>
       <c r="F50" s="275" t="n"/>
@@ -4130,23 +4130,22 @@
       <c r="N50" s="275" t="n"/>
       <c r="O50" s="275" t="n"/>
       <c r="P50" s="270" t="n"/>
-      <c r="Q50" s="1" t="n"/>
-      <c r="R50" s="1" t="n"/>
-    </row>
-    <row r="51" ht="18.75" customHeight="1">
-      <c r="A51" s="1" t="n"/>
+      <c r="Q50" s="13" t="n"/>
+      <c r="R50" s="13" t="n"/>
+    </row>
+    <row r="51" ht="22.5" customHeight="1">
       <c r="B51" s="297" t="n"/>
       <c r="C51" s="141" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D51" s="22" t="inlineStr">
         <is>
-          <t>@@ACT7_DIAS@@</t>
+          <t>@@ACT5_DIAS@@</t>
         </is>
       </c>
       <c r="E51" s="151" t="inlineStr">
         <is>
-          <t>@@ACT7_DESC@@</t>
+          <t>@@ACT5_DESC@@</t>
         </is>
       </c>
       <c r="F51" s="275" t="n"/>
@@ -4160,156 +4159,139 @@
       <c r="N51" s="275" t="n"/>
       <c r="O51" s="275" t="n"/>
       <c r="P51" s="270" t="n"/>
-    </row>
-    <row r="52" ht="24" customHeight="1" thickBot="1">
-      <c r="A52" s="1" t="n"/>
-      <c r="B52" s="88" t="n"/>
-      <c r="C52" s="139" t="n">
+      <c r="Q51" s="13" t="n"/>
+      <c r="R51" s="13" t="n"/>
+    </row>
+    <row r="52" ht="18.75" customHeight="1" thickBot="1">
+      <c r="B52" s="297" t="n"/>
+      <c r="C52" s="141" t="n">
+        <v>6</v>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT6_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E52" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT6_DESC@@</t>
+        </is>
+      </c>
+      <c r="F52" s="275" t="n"/>
+      <c r="G52" s="275" t="n"/>
+      <c r="H52" s="275" t="n"/>
+      <c r="I52" s="275" t="n"/>
+      <c r="J52" s="275" t="n"/>
+      <c r="K52" s="275" t="n"/>
+      <c r="L52" s="275" t="n"/>
+      <c r="M52" s="275" t="n"/>
+      <c r="N52" s="275" t="n"/>
+      <c r="O52" s="275" t="n"/>
+      <c r="P52" s="270" t="n"/>
+      <c r="Q52" s="1" t="n"/>
+      <c r="R52" s="1" t="n"/>
+    </row>
+    <row r="53" ht="18.75" customHeight="1" thickBot="1">
+      <c r="A53" s="1" t="n"/>
+      <c r="B53" s="297" t="n"/>
+      <c r="C53" s="141" t="n">
+        <v>7</v>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT7_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E53" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT7_DESC@@</t>
+        </is>
+      </c>
+      <c r="F53" s="275" t="n"/>
+      <c r="G53" s="275" t="n"/>
+      <c r="H53" s="275" t="n"/>
+      <c r="I53" s="275" t="n"/>
+      <c r="J53" s="275" t="n"/>
+      <c r="K53" s="275" t="n"/>
+      <c r="L53" s="275" t="n"/>
+      <c r="M53" s="275" t="n"/>
+      <c r="N53" s="275" t="n"/>
+      <c r="O53" s="275" t="n"/>
+      <c r="P53" s="270" t="n"/>
+    </row>
+    <row r="54" ht="24" customHeight="1" thickBot="1">
+      <c r="A54" s="1" t="n"/>
+      <c r="B54" s="297" t="n"/>
+      <c r="C54" s="139" t="n">
         <v>8</v>
       </c>
-      <c r="D52" s="30" t="inlineStr">
+      <c r="D54" s="30" t="inlineStr">
         <is>
           <t>@@ACT8_DIAS@@</t>
         </is>
       </c>
-      <c r="E52" s="198" t="inlineStr">
+      <c r="E54" s="198" t="inlineStr">
         <is>
           <t>@@ACT8_DESC@@</t>
         </is>
       </c>
-      <c r="F52" s="276" t="n"/>
-      <c r="G52" s="276" t="n"/>
-      <c r="H52" s="276" t="n"/>
-      <c r="I52" s="276" t="n"/>
-      <c r="J52" s="276" t="n"/>
-      <c r="K52" s="276" t="n"/>
-      <c r="L52" s="276" t="n"/>
-      <c r="M52" s="276" t="n"/>
-      <c r="N52" s="276" t="n"/>
-      <c r="O52" s="276" t="n"/>
-      <c r="P52" s="271" t="n"/>
-    </row>
-    <row r="53" ht="24" customHeight="1" thickBot="1">
-      <c r="A53" s="1" t="n"/>
-      <c r="B53" s="4" t="n"/>
-      <c r="C53" s="1" t="n"/>
-      <c r="D53" s="1" t="n"/>
-      <c r="E53" s="1" t="n"/>
-      <c r="F53" s="1" t="n"/>
-      <c r="G53" s="1" t="n"/>
-      <c r="H53" s="1" t="n"/>
-      <c r="I53" s="1" t="n"/>
-      <c r="J53" s="1" t="n"/>
-      <c r="K53" s="1" t="n"/>
-      <c r="L53" s="1" t="n"/>
-      <c r="M53" s="1" t="n"/>
-      <c r="N53" s="1" t="n"/>
-      <c r="O53" s="1" t="n"/>
-      <c r="P53" s="1" t="n"/>
-    </row>
-    <row r="54" ht="128.25" customHeight="1" thickBot="1">
-      <c r="A54" s="1" t="n"/>
-      <c r="B54" s="108" t="inlineStr">
-        <is>
-          <t>Nombre Funcionario</t>
-        </is>
-      </c>
-      <c r="C54" s="109" t="inlineStr">
-        <is>
-          <t>Elementos de Protección Personal asignado</t>
-        </is>
-      </c>
-      <c r="D54" s="110" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="E54" s="229" t="inlineStr">
-        <is>
-          <t>Estado del EPP</t>
-        </is>
-      </c>
-      <c r="F54" s="218" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-      <c r="G54" s="84" t="n"/>
-      <c r="H54" s="84" t="n"/>
-      <c r="I54" s="84" t="n"/>
-      <c r="J54" s="84" t="n"/>
-      <c r="K54" s="84" t="n"/>
-      <c r="L54" s="84" t="n"/>
-      <c r="M54" s="84" t="n"/>
-      <c r="N54" s="84" t="n"/>
-      <c r="O54" s="84" t="n"/>
-      <c r="P54" s="253" t="n"/>
+      <c r="F54" s="276" t="n"/>
+      <c r="G54" s="276" t="n"/>
+      <c r="H54" s="276" t="n"/>
+      <c r="I54" s="276" t="n"/>
+      <c r="J54" s="276" t="n"/>
+      <c r="K54" s="276" t="n"/>
+      <c r="L54" s="276" t="n"/>
+      <c r="M54" s="276" t="n"/>
+      <c r="N54" s="276" t="n"/>
+      <c r="O54" s="276" t="n"/>
+      <c r="P54" s="271" t="n"/>
     </row>
     <row r="55" ht="18.75" customHeight="1">
       <c r="A55" s="1" t="n"/>
-      <c r="B55" s="107" t="inlineStr">
-        <is>
-          <t>@@EPP1_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C55" s="71" t="inlineStr">
-        <is>
-          <t>@@EPP1_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D55" s="103" t="inlineStr">
-        <is>
-          <t>@@EPP1_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E55" s="103" t="inlineStr">
-        <is>
-          <t>@@EPP1_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F55" s="298" t="inlineStr">
-        <is>
-          <t>@@EPP1_OBS@@</t>
-        </is>
-      </c>
-      <c r="G55" s="257" t="n"/>
-      <c r="H55" s="257" t="n"/>
-      <c r="I55" s="257" t="n"/>
-      <c r="J55" s="257" t="n"/>
-      <c r="K55" s="257" t="n"/>
-      <c r="L55" s="257" t="n"/>
-      <c r="M55" s="257" t="n"/>
-      <c r="N55" s="257" t="n"/>
-      <c r="O55" s="257" t="n"/>
-      <c r="P55" s="299" t="n"/>
+      <c r="B55" s="297" t="n"/>
+      <c r="C55" s="141" t="n">
+        <v>9</v>
+      </c>
+      <c r="D55" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT9_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E55" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT9_DESC@@</t>
+        </is>
+      </c>
+      <c r="F55" s="275" t="n"/>
+      <c r="G55" s="275" t="n"/>
+      <c r="H55" s="275" t="n"/>
+      <c r="I55" s="275" t="n"/>
+      <c r="J55" s="275" t="n"/>
+      <c r="K55" s="275" t="n"/>
+      <c r="L55" s="275" t="n"/>
+      <c r="M55" s="275" t="n"/>
+      <c r="N55" s="275" t="n"/>
+      <c r="O55" s="275" t="n"/>
+      <c r="P55" s="270" t="n"/>
     </row>
     <row r="56" ht="18.75" customHeight="1">
       <c r="A56" s="1" t="n"/>
-      <c r="B56" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP2_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C56" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP2_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D56" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP2_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E56" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP2_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F56" s="166" t="inlineStr">
-        <is>
-          <t>@@EPP2_OBS@@</t>
-        </is>
-      </c>
+      <c r="B56" s="297" t="n"/>
+      <c r="C56" s="141" t="n">
+        <v>10</v>
+      </c>
+      <c r="D56" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT10_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E56" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT10_DESC@@</t>
+        </is>
+      </c>
+      <c r="F56" s="275" t="n"/>
       <c r="G56" s="275" t="n"/>
       <c r="H56" s="275" t="n"/>
       <c r="I56" s="275" t="n"/>
@@ -4319,35 +4301,25 @@
       <c r="M56" s="275" t="n"/>
       <c r="N56" s="275" t="n"/>
       <c r="O56" s="275" t="n"/>
-      <c r="P56" s="279" t="n"/>
+      <c r="P56" s="270" t="n"/>
     </row>
     <row r="57" ht="18.75" customHeight="1">
       <c r="A57" s="1" t="n"/>
-      <c r="B57" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP3_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C57" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP3_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP3_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E57" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP3_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F57" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP3_OBS@@</t>
-        </is>
-      </c>
+      <c r="B57" s="297" t="n"/>
+      <c r="C57" s="141" t="n">
+        <v>11</v>
+      </c>
+      <c r="D57" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT11_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E57" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT11_DESC@@</t>
+        </is>
+      </c>
+      <c r="F57" s="275" t="n"/>
       <c r="G57" s="275" t="n"/>
       <c r="H57" s="275" t="n"/>
       <c r="I57" s="275" t="n"/>
@@ -4361,31 +4333,21 @@
     </row>
     <row r="58" ht="18.75" customHeight="1">
       <c r="A58" s="1" t="n"/>
-      <c r="B58" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP4_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C58" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP4_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D58" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP4_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E58" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP4_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F58" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP4_OBS@@</t>
-        </is>
-      </c>
+      <c r="B58" s="297" t="n"/>
+      <c r="C58" s="141" t="n">
+        <v>12</v>
+      </c>
+      <c r="D58" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT12_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E58" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT12_DESC@@</t>
+        </is>
+      </c>
+      <c r="F58" s="275" t="n"/>
       <c r="G58" s="275" t="n"/>
       <c r="H58" s="275" t="n"/>
       <c r="I58" s="275" t="n"/>
@@ -4398,31 +4360,22 @@
       <c r="P58" s="270" t="n"/>
     </row>
     <row r="59" ht="18.75" customHeight="1">
-      <c r="B59" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP5_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C59" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP5_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP5_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E59" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP5_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F59" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP5_OBS@@</t>
-        </is>
-      </c>
+      <c r="A59" s="1" t="n"/>
+      <c r="B59" s="297" t="n"/>
+      <c r="C59" s="141" t="n">
+        <v>13</v>
+      </c>
+      <c r="D59" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT13_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E59" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT13_DESC@@</t>
+        </is>
+      </c>
+      <c r="F59" s="275" t="n"/>
       <c r="G59" s="275" t="n"/>
       <c r="H59" s="275" t="n"/>
       <c r="I59" s="275" t="n"/>
@@ -4435,31 +4388,22 @@
       <c r="P59" s="270" t="n"/>
     </row>
     <row r="60" ht="18.75" customHeight="1">
-      <c r="B60" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP6_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C60" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP6_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP6_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E60" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP6_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F60" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP6_OBS@@</t>
-        </is>
-      </c>
+      <c r="A60" s="1" t="n"/>
+      <c r="B60" s="88" t="n"/>
+      <c r="C60" s="141" t="n">
+        <v>14</v>
+      </c>
+      <c r="D60" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT14_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E60" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT14_DESC@@</t>
+        </is>
+      </c>
+      <c r="F60" s="275" t="n"/>
       <c r="G60" s="275" t="n"/>
       <c r="H60" s="275" t="n"/>
       <c r="I60" s="275" t="n"/>
@@ -4471,463 +4415,770 @@
       <c r="O60" s="275" t="n"/>
       <c r="P60" s="270" t="n"/>
     </row>
-    <row r="61" ht="18.75" customHeight="1">
-      <c r="B61" s="24" t="inlineStr">
+    <row r="61" ht="24" customHeight="1">
+      <c r="A61" s="1" t="n"/>
+      <c r="B61" s="4" t="n"/>
+      <c r="C61" s="1" t="n"/>
+      <c r="D61" s="1" t="n"/>
+      <c r="E61" s="1" t="n"/>
+      <c r="F61" s="1" t="n"/>
+      <c r="G61" s="1" t="n"/>
+      <c r="H61" s="1" t="n"/>
+      <c r="I61" s="1" t="n"/>
+      <c r="J61" s="1" t="n"/>
+      <c r="K61" s="1" t="n"/>
+      <c r="L61" s="1" t="n"/>
+      <c r="M61" s="1" t="n"/>
+      <c r="N61" s="1" t="n"/>
+      <c r="O61" s="1" t="n"/>
+      <c r="P61" s="1" t="n"/>
+    </row>
+    <row r="62" ht="128.25" customHeight="1">
+      <c r="A62" s="1" t="n"/>
+      <c r="B62" s="108" t="inlineStr">
+        <is>
+          <t>Nombre Funcionario</t>
+        </is>
+      </c>
+      <c r="C62" s="109" t="inlineStr">
+        <is>
+          <t>Elementos de Protección Personal asignado</t>
+        </is>
+      </c>
+      <c r="D62" s="110" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E62" s="229" t="inlineStr">
+        <is>
+          <t>Estado del EPP</t>
+        </is>
+      </c>
+      <c r="F62" s="218" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="G62" s="84" t="n"/>
+      <c r="H62" s="84" t="n"/>
+      <c r="I62" s="84" t="n"/>
+      <c r="J62" s="84" t="n"/>
+      <c r="K62" s="84" t="n"/>
+      <c r="L62" s="84" t="n"/>
+      <c r="M62" s="84" t="n"/>
+      <c r="N62" s="84" t="n"/>
+      <c r="O62" s="84" t="n"/>
+      <c r="P62" s="253" t="n"/>
+    </row>
+    <row r="63" ht="18.75" customHeight="1">
+      <c r="A63" s="1" t="n"/>
+      <c r="B63" s="107" t="inlineStr">
+        <is>
+          <t>@@EPP1_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C63" s="71" t="inlineStr">
+        <is>
+          <t>@@EPP1_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D63" s="103" t="inlineStr">
+        <is>
+          <t>@@EPP1_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E63" s="103" t="inlineStr">
+        <is>
+          <t>@@EPP1_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F63" s="298" t="inlineStr">
+        <is>
+          <t>@@EPP1_OBS@@</t>
+        </is>
+      </c>
+      <c r="G63" s="257" t="n"/>
+      <c r="H63" s="257" t="n"/>
+      <c r="I63" s="257" t="n"/>
+      <c r="J63" s="257" t="n"/>
+      <c r="K63" s="257" t="n"/>
+      <c r="L63" s="257" t="n"/>
+      <c r="M63" s="257" t="n"/>
+      <c r="N63" s="257" t="n"/>
+      <c r="O63" s="257" t="n"/>
+      <c r="P63" s="299" t="n"/>
+    </row>
+    <row r="64" ht="18.75" customHeight="1" thickBot="1">
+      <c r="A64" s="1" t="n"/>
+      <c r="B64" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP2_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C64" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP2_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP2_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E64" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP2_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F64" s="166" t="inlineStr">
+        <is>
+          <t>@@EPP2_OBS@@</t>
+        </is>
+      </c>
+      <c r="G64" s="275" t="n"/>
+      <c r="H64" s="275" t="n"/>
+      <c r="I64" s="275" t="n"/>
+      <c r="J64" s="275" t="n"/>
+      <c r="K64" s="275" t="n"/>
+      <c r="L64" s="275" t="n"/>
+      <c r="M64" s="275" t="n"/>
+      <c r="N64" s="275" t="n"/>
+      <c r="O64" s="275" t="n"/>
+      <c r="P64" s="279" t="n"/>
+    </row>
+    <row r="65" ht="18.75" customHeight="1">
+      <c r="A65" s="1" t="n"/>
+      <c r="B65" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP3_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C65" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP3_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP3_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E65" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP3_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F65" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP3_OBS@@</t>
+        </is>
+      </c>
+      <c r="G65" s="275" t="n"/>
+      <c r="H65" s="275" t="n"/>
+      <c r="I65" s="275" t="n"/>
+      <c r="J65" s="275" t="n"/>
+      <c r="K65" s="275" t="n"/>
+      <c r="L65" s="275" t="n"/>
+      <c r="M65" s="275" t="n"/>
+      <c r="N65" s="275" t="n"/>
+      <c r="O65" s="275" t="n"/>
+      <c r="P65" s="270" t="n"/>
+    </row>
+    <row r="66" ht="18.75" customHeight="1" thickBot="1">
+      <c r="A66" s="1" t="n"/>
+      <c r="B66" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP4_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C66" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP4_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP4_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E66" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP4_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F66" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP4_OBS@@</t>
+        </is>
+      </c>
+      <c r="G66" s="275" t="n"/>
+      <c r="H66" s="275" t="n"/>
+      <c r="I66" s="275" t="n"/>
+      <c r="J66" s="275" t="n"/>
+      <c r="K66" s="275" t="n"/>
+      <c r="L66" s="275" t="n"/>
+      <c r="M66" s="275" t="n"/>
+      <c r="N66" s="275" t="n"/>
+      <c r="O66" s="275" t="n"/>
+      <c r="P66" s="270" t="n"/>
+    </row>
+    <row r="67" ht="18.75" customHeight="1">
+      <c r="B67" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP5_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C67" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP5_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP5_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E67" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP5_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F67" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP5_OBS@@</t>
+        </is>
+      </c>
+      <c r="G67" s="275" t="n"/>
+      <c r="H67" s="275" t="n"/>
+      <c r="I67" s="275" t="n"/>
+      <c r="J67" s="275" t="n"/>
+      <c r="K67" s="275" t="n"/>
+      <c r="L67" s="275" t="n"/>
+      <c r="M67" s="275" t="n"/>
+      <c r="N67" s="275" t="n"/>
+      <c r="O67" s="275" t="n"/>
+      <c r="P67" s="270" t="n"/>
+    </row>
+    <row r="68" ht="18.75" customHeight="1">
+      <c r="B68" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP6_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C68" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP6_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP6_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E68" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP6_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F68" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP6_OBS@@</t>
+        </is>
+      </c>
+      <c r="G68" s="275" t="n"/>
+      <c r="H68" s="275" t="n"/>
+      <c r="I68" s="275" t="n"/>
+      <c r="J68" s="275" t="n"/>
+      <c r="K68" s="275" t="n"/>
+      <c r="L68" s="275" t="n"/>
+      <c r="M68" s="275" t="n"/>
+      <c r="N68" s="275" t="n"/>
+      <c r="O68" s="275" t="n"/>
+      <c r="P68" s="270" t="n"/>
+    </row>
+    <row r="69" ht="18.75" customHeight="1">
+      <c r="B69" s="24" t="inlineStr">
         <is>
           <t>@@EPP7_NOMBRE@@</t>
         </is>
       </c>
-      <c r="C61" s="141" t="inlineStr">
+      <c r="C69" s="141" t="inlineStr">
         <is>
           <t>@@EPP7_ELEMENTO@@</t>
         </is>
       </c>
-      <c r="D61" s="21" t="inlineStr">
+      <c r="D69" s="21" t="inlineStr">
         <is>
           <t>@@EPP7_CANTIDAD@@</t>
         </is>
       </c>
-      <c r="E61" s="21" t="inlineStr">
+      <c r="E69" s="21" t="inlineStr">
         <is>
           <t>@@EPP7_ESTADO@@</t>
         </is>
       </c>
-      <c r="F61" s="165" t="inlineStr">
+      <c r="F69" s="165" t="inlineStr">
         <is>
           <t>@@EPP7_OBS@@</t>
         </is>
       </c>
-      <c r="G61" s="275" t="n"/>
-      <c r="H61" s="275" t="n"/>
-      <c r="I61" s="275" t="n"/>
-      <c r="J61" s="275" t="n"/>
-      <c r="K61" s="275" t="n"/>
-      <c r="L61" s="275" t="n"/>
-      <c r="M61" s="275" t="n"/>
-      <c r="N61" s="275" t="n"/>
-      <c r="O61" s="275" t="n"/>
-      <c r="P61" s="270" t="n"/>
-    </row>
-    <row r="62" ht="18.75" customHeight="1">
-      <c r="B62" s="24" t="inlineStr">
+      <c r="G69" s="275" t="n"/>
+      <c r="H69" s="275" t="n"/>
+      <c r="I69" s="275" t="n"/>
+      <c r="J69" s="275" t="n"/>
+      <c r="K69" s="275" t="n"/>
+      <c r="L69" s="275" t="n"/>
+      <c r="M69" s="275" t="n"/>
+      <c r="N69" s="275" t="n"/>
+      <c r="O69" s="275" t="n"/>
+      <c r="P69" s="270" t="n"/>
+    </row>
+    <row r="70" ht="18.75" customHeight="1" thickBot="1">
+      <c r="B70" s="24" t="inlineStr">
         <is>
           <t>@@EPP8_NOMBRE@@</t>
         </is>
       </c>
-      <c r="C62" s="141" t="inlineStr">
+      <c r="C70" s="141" t="inlineStr">
         <is>
           <t>@@EPP8_ELEMENTO@@</t>
         </is>
       </c>
-      <c r="D62" s="21" t="inlineStr">
+      <c r="D70" s="21" t="inlineStr">
         <is>
           <t>@@EPP8_CANTIDAD@@</t>
         </is>
       </c>
-      <c r="E62" s="21" t="inlineStr">
+      <c r="E70" s="21" t="inlineStr">
         <is>
           <t>@@EPP8_ESTADO@@</t>
         </is>
       </c>
-      <c r="F62" s="165" t="inlineStr">
+      <c r="F70" s="165" t="inlineStr">
         <is>
           <t>@@EPP8_OBS@@</t>
         </is>
       </c>
-      <c r="G62" s="275" t="n"/>
-      <c r="H62" s="275" t="n"/>
-      <c r="I62" s="275" t="n"/>
-      <c r="J62" s="275" t="n"/>
-      <c r="K62" s="275" t="n"/>
-      <c r="L62" s="275" t="n"/>
-      <c r="M62" s="275" t="n"/>
-      <c r="N62" s="275" t="n"/>
-      <c r="O62" s="275" t="n"/>
-      <c r="P62" s="270" t="n"/>
-    </row>
-    <row r="63" ht="18.75" customHeight="1">
-      <c r="B63" s="24" t="inlineStr">
+      <c r="G70" s="275" t="n"/>
+      <c r="H70" s="275" t="n"/>
+      <c r="I70" s="275" t="n"/>
+      <c r="J70" s="275" t="n"/>
+      <c r="K70" s="275" t="n"/>
+      <c r="L70" s="275" t="n"/>
+      <c r="M70" s="275" t="n"/>
+      <c r="N70" s="275" t="n"/>
+      <c r="O70" s="275" t="n"/>
+      <c r="P70" s="270" t="n"/>
+    </row>
+    <row r="71" ht="18.75" customHeight="1">
+      <c r="B71" s="24" t="inlineStr">
         <is>
           <t>@@EPP9_NOMBRE@@</t>
         </is>
       </c>
-      <c r="C63" s="141" t="inlineStr">
+      <c r="C71" s="141" t="inlineStr">
         <is>
           <t>@@EPP9_ELEMENTO@@</t>
         </is>
       </c>
-      <c r="D63" s="21" t="inlineStr">
+      <c r="D71" s="21" t="inlineStr">
         <is>
           <t>@@EPP9_CANTIDAD@@</t>
         </is>
       </c>
-      <c r="E63" s="21" t="inlineStr">
+      <c r="E71" s="21" t="inlineStr">
         <is>
           <t>@@EPP9_ESTADO@@</t>
         </is>
       </c>
-      <c r="F63" s="165" t="inlineStr">
+      <c r="F71" s="165" t="inlineStr">
         <is>
           <t>@@EPP9_OBS@@</t>
         </is>
       </c>
-      <c r="G63" s="275" t="n"/>
-      <c r="H63" s="275" t="n"/>
-      <c r="I63" s="275" t="n"/>
-      <c r="J63" s="275" t="n"/>
-      <c r="K63" s="275" t="n"/>
-      <c r="L63" s="275" t="n"/>
-      <c r="M63" s="275" t="n"/>
-      <c r="N63" s="275" t="n"/>
-      <c r="O63" s="275" t="n"/>
-      <c r="P63" s="270" t="n"/>
-    </row>
-    <row r="64" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B64" s="98" t="inlineStr">
+      <c r="G71" s="275" t="n"/>
+      <c r="H71" s="275" t="n"/>
+      <c r="I71" s="275" t="n"/>
+      <c r="J71" s="275" t="n"/>
+      <c r="K71" s="275" t="n"/>
+      <c r="L71" s="275" t="n"/>
+      <c r="M71" s="275" t="n"/>
+      <c r="N71" s="275" t="n"/>
+      <c r="O71" s="275" t="n"/>
+      <c r="P71" s="270" t="n"/>
+    </row>
+    <row r="72" ht="19.5" customHeight="1">
+      <c r="B72" s="98" t="inlineStr">
         <is>
           <t>@@EPP10_NOMBRE@@</t>
         </is>
       </c>
-      <c r="C64" s="139" t="inlineStr">
+      <c r="C72" s="139" t="inlineStr">
         <is>
           <t>@@EPP10_ELEMENTO@@</t>
         </is>
       </c>
-      <c r="D64" s="99" t="inlineStr">
+      <c r="D72" s="99" t="inlineStr">
         <is>
           <t>@@EPP10_CANTIDAD@@</t>
         </is>
       </c>
-      <c r="E64" s="99" t="inlineStr">
+      <c r="E72" s="99" t="inlineStr">
         <is>
           <t>@@EPP10_ESTADO@@</t>
         </is>
       </c>
-      <c r="F64" s="167" t="inlineStr">
+      <c r="F72" s="167" t="inlineStr">
         <is>
           <t>@@EPP10_OBS@@</t>
         </is>
       </c>
-      <c r="G64" s="276" t="n"/>
-      <c r="H64" s="276" t="n"/>
-      <c r="I64" s="276" t="n"/>
-      <c r="J64" s="276" t="n"/>
-      <c r="K64" s="276" t="n"/>
-      <c r="L64" s="276" t="n"/>
-      <c r="M64" s="276" t="n"/>
-      <c r="N64" s="276" t="n"/>
-      <c r="O64" s="276" t="n"/>
-      <c r="P64" s="271" t="n"/>
-    </row>
-    <row r="66" ht="15.75" customHeight="1" thickBot="1"/>
-    <row r="67" ht="18.75" customHeight="1">
-      <c r="B67" s="300" t="inlineStr">
+      <c r="G72" s="276" t="n"/>
+      <c r="H72" s="276" t="n"/>
+      <c r="I72" s="276" t="n"/>
+      <c r="J72" s="276" t="n"/>
+      <c r="K72" s="276" t="n"/>
+      <c r="L72" s="276" t="n"/>
+      <c r="M72" s="276" t="n"/>
+      <c r="N72" s="276" t="n"/>
+      <c r="O72" s="276" t="n"/>
+      <c r="P72" s="271" t="n"/>
+    </row>
+    <row r="73"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="18.75" customHeight="1">
+      <c r="B75" s="300" t="inlineStr">
         <is>
           <t>Seguridad y Riesgos</t>
         </is>
       </c>
-      <c r="C67" s="273" t="n"/>
-      <c r="D67" s="273" t="n"/>
-      <c r="E67" s="274" t="n"/>
-    </row>
-    <row r="68" ht="18.75" customHeight="1">
-      <c r="B68" s="17" t="inlineStr">
+      <c r="C75" s="273" t="n"/>
+      <c r="D75" s="273" t="n"/>
+      <c r="E75" s="274" t="n"/>
+    </row>
+    <row r="76" ht="18.75" customHeight="1">
+      <c r="B76" s="17" t="inlineStr">
         <is>
           <t>Identificación de riesgos</t>
         </is>
       </c>
-      <c r="C68" s="166" t="inlineStr">
+      <c r="C76" s="166" t="inlineStr">
         <is>
           <t>@@RIESGOS_IDENT@@</t>
         </is>
       </c>
-      <c r="D68" s="275" t="n"/>
-      <c r="E68" s="279" t="n"/>
-    </row>
-    <row r="69" ht="18.75" customHeight="1">
-      <c r="B69" s="17" t="inlineStr">
+      <c r="D76" s="275" t="n"/>
+      <c r="E76" s="279" t="n"/>
+    </row>
+    <row r="77" ht="18.75" customHeight="1">
+      <c r="B77" s="17" t="inlineStr">
         <is>
           <t>Medidas preventivas</t>
         </is>
       </c>
-      <c r="C69" s="166" t="inlineStr">
+      <c r="C77" s="166" t="inlineStr">
         <is>
           <t>@@RIESGOS_MEDIDAS@@</t>
         </is>
       </c>
-      <c r="D69" s="275" t="n"/>
-      <c r="E69" s="279" t="n"/>
-    </row>
-    <row r="70" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B70" s="18" t="inlineStr">
+      <c r="D77" s="275" t="n"/>
+      <c r="E77" s="279" t="n"/>
+    </row>
+    <row r="78" ht="19.5" customHeight="1">
+      <c r="B78" s="18" t="inlineStr">
         <is>
           <t>Plan de emergencia</t>
         </is>
       </c>
-      <c r="C70" s="168" t="inlineStr">
+      <c r="C78" s="168" t="inlineStr">
         <is>
           <t>@@RIESGOS_PLAN_EMERG@@</t>
         </is>
       </c>
-      <c r="D70" s="276" t="n"/>
-      <c r="E70" s="301" t="n"/>
-    </row>
-    <row r="73" ht="18.75" customHeight="1">
-      <c r="B73" s="58" t="n"/>
-      <c r="C73" s="67" t="inlineStr">
+      <c r="D78" s="276" t="n"/>
+      <c r="E78" s="301" t="n"/>
+    </row>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81" ht="18.75" customHeight="1">
+      <c r="B81" s="58" t="n"/>
+      <c r="C81" s="67" t="inlineStr">
         <is>
           <t>Día</t>
         </is>
       </c>
-      <c r="D73" s="67" t="inlineStr">
+      <c r="D81" s="67" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="E73" s="67" t="inlineStr">
+      <c r="E81" s="67" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="F73" s="51" t="n"/>
-      <c r="G73" s="51" t="n"/>
-      <c r="H73" s="51" t="n"/>
-      <c r="I73" s="51" t="n"/>
-      <c r="J73" s="51" t="n"/>
-      <c r="K73" s="51" t="n"/>
-    </row>
-    <row r="74" ht="18.75" customHeight="1">
-      <c r="B74" s="52" t="inlineStr">
-        <is>
-          <t>FECHA ELABORACIÓN:</t>
-        </is>
-      </c>
-      <c r="C74" s="57" t="inlineStr">
-        <is>
-          <t>@@ELAB_DIA@@</t>
-        </is>
-      </c>
-      <c r="D74" s="57" t="inlineStr">
-        <is>
-          <t>@@ELAB_MES@@</t>
-        </is>
-      </c>
-      <c r="E74" s="53" t="inlineStr">
-        <is>
-          <t>@@ELAB_ANIO@@</t>
-        </is>
-      </c>
-      <c r="F74" s="50" t="n"/>
-      <c r="G74" s="51" t="n"/>
-      <c r="H74" s="51" t="n"/>
-      <c r="I74" s="51" t="n"/>
-      <c r="J74" s="51" t="n"/>
-      <c r="K74" s="51" t="n"/>
-    </row>
-    <row r="75" ht="18.75" customHeight="1">
-      <c r="B75" s="52" t="inlineStr">
-        <is>
-          <t>ELABORADO POR:</t>
-        </is>
-      </c>
-      <c r="C75" s="302" t="inlineStr">
-        <is>
-          <t>@@ELABORADO_POR@@</t>
-        </is>
-      </c>
-      <c r="D75" s="275" t="n"/>
-      <c r="E75" s="270" t="n"/>
-      <c r="F75" s="173" t="inlineStr">
-        <is>
-          <t>FIRMA (JEFE PROYECTO)</t>
-        </is>
-      </c>
-      <c r="H75" s="51" t="n"/>
-      <c r="I75" s="51" t="n"/>
-      <c r="J75" s="51" t="n"/>
-      <c r="K75" s="51" t="n"/>
-    </row>
-    <row r="76" ht="18.75" customHeight="1">
-      <c r="B76" s="55" t="n"/>
-      <c r="C76" s="54" t="n"/>
-      <c r="D76" s="54" t="n"/>
-      <c r="E76" s="54" t="n"/>
-      <c r="F76" s="51" t="n"/>
-      <c r="G76" s="51" t="n"/>
-      <c r="H76" s="51" t="n"/>
-      <c r="I76" s="51" t="n"/>
-      <c r="J76" s="51" t="n"/>
-      <c r="K76" s="51" t="n"/>
-    </row>
-    <row r="77" ht="18.75" customHeight="1"/>
-    <row r="78" ht="18.75" customHeight="1">
-      <c r="B78" s="55" t="n"/>
-      <c r="C78" s="174" t="n"/>
-      <c r="D78" s="174" t="n"/>
-      <c r="E78" s="174" t="n"/>
-      <c r="F78" s="51" t="n"/>
-      <c r="G78" s="51" t="n"/>
-      <c r="H78" s="51" t="n"/>
-      <c r="I78" s="51" t="n"/>
-      <c r="J78" s="51" t="n"/>
-      <c r="K78" s="51" t="n"/>
-    </row>
-    <row r="79" ht="18.75" customHeight="1">
-      <c r="B79" s="58" t="n"/>
-      <c r="C79" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_DIA@@</t>
-        </is>
-      </c>
-      <c r="D79" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_MES@@</t>
-        </is>
-      </c>
-      <c r="E79" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_ANIO@@</t>
-        </is>
-      </c>
-      <c r="F79" s="51" t="n"/>
-      <c r="G79" s="51" t="n"/>
-      <c r="H79" s="51" t="n"/>
-      <c r="I79" s="51" t="n"/>
-      <c r="J79" s="51" t="n"/>
-      <c r="K79" s="51" t="n"/>
-    </row>
-    <row r="80" ht="18.75" customHeight="1">
-      <c r="B80" s="52" t="inlineStr">
-        <is>
-          <t>FECHA REVISIÓN:</t>
-        </is>
-      </c>
-      <c r="C80" s="57" t="n"/>
-      <c r="D80" s="57" t="n"/>
-      <c r="E80" s="53" t="n"/>
-      <c r="F80" s="51" t="n"/>
-      <c r="G80" s="51" t="n"/>
-      <c r="H80" s="51" t="n"/>
-      <c r="I80" s="51" t="n"/>
-      <c r="J80" s="51" t="n"/>
-      <c r="K80" s="51" t="n"/>
-    </row>
-    <row r="81" ht="18.75" customHeight="1">
-      <c r="B81" s="52" t="inlineStr">
-        <is>
-          <t>REVISADO  POR:</t>
-        </is>
-      </c>
-      <c r="C81" s="302" t="inlineStr">
-        <is>
-          <t>@@REVISADO_POR@@</t>
-        </is>
-      </c>
-      <c r="D81" s="275" t="n"/>
-      <c r="E81" s="270" t="n"/>
-      <c r="F81" s="173" t="inlineStr">
-        <is>
-          <t>FIRMA (JEFE DEPARTAMENTO)</t>
-        </is>
-      </c>
+      <c r="F81" s="51" t="n"/>
+      <c r="G81" s="51" t="n"/>
       <c r="H81" s="51" t="n"/>
       <c r="I81" s="51" t="n"/>
       <c r="J81" s="51" t="n"/>
       <c r="K81" s="51" t="n"/>
     </row>
+    <row r="82" ht="18.75" customHeight="1">
+      <c r="B82" s="52" t="inlineStr">
+        <is>
+          <t>FECHA ELABORACIÓN:</t>
+        </is>
+      </c>
+      <c r="C82" s="57" t="inlineStr">
+        <is>
+          <t>@@ELAB_DIA@@</t>
+        </is>
+      </c>
+      <c r="D82" s="57" t="inlineStr">
+        <is>
+          <t>@@ELAB_MES@@</t>
+        </is>
+      </c>
+      <c r="E82" s="53" t="inlineStr">
+        <is>
+          <t>@@ELAB_ANIO@@</t>
+        </is>
+      </c>
+      <c r="F82" s="50" t="n"/>
+      <c r="G82" s="51" t="n"/>
+      <c r="H82" s="51" t="n"/>
+      <c r="I82" s="51" t="n"/>
+      <c r="J82" s="51" t="n"/>
+      <c r="K82" s="51" t="n"/>
+    </row>
+    <row r="83" ht="18.75" customHeight="1">
+      <c r="B83" s="52" t="inlineStr">
+        <is>
+          <t>ELABORADO POR:</t>
+        </is>
+      </c>
+      <c r="C83" s="302" t="inlineStr">
+        <is>
+          <t>@@ELABORADO_POR@@</t>
+        </is>
+      </c>
+      <c r="D83" s="275" t="n"/>
+      <c r="E83" s="270" t="n"/>
+      <c r="F83" s="173" t="inlineStr">
+        <is>
+          <t>FIRMA (JEFE PROYECTO)</t>
+        </is>
+      </c>
+      <c r="H83" s="51" t="n"/>
+      <c r="I83" s="51" t="n"/>
+      <c r="J83" s="51" t="n"/>
+      <c r="K83" s="51" t="n"/>
+    </row>
+    <row r="84" ht="18.75" customHeight="1">
+      <c r="B84" s="55" t="n"/>
+      <c r="C84" s="54" t="n"/>
+      <c r="D84" s="54" t="n"/>
+      <c r="E84" s="54" t="n"/>
+      <c r="F84" s="51" t="n"/>
+      <c r="G84" s="51" t="n"/>
+      <c r="H84" s="51" t="n"/>
+      <c r="I84" s="51" t="n"/>
+      <c r="J84" s="51" t="n"/>
+      <c r="K84" s="51" t="n"/>
+    </row>
+    <row r="85" ht="18.75" customHeight="1"/>
     <row r="86" ht="18.75" customHeight="1">
-      <c r="B86" s="169" t="inlineStr">
+      <c r="B86" s="55" t="n"/>
+      <c r="C86" s="174" t="n"/>
+      <c r="D86" s="174" t="n"/>
+      <c r="E86" s="174" t="n"/>
+      <c r="F86" s="51" t="n"/>
+      <c r="G86" s="51" t="n"/>
+      <c r="H86" s="51" t="n"/>
+      <c r="I86" s="51" t="n"/>
+      <c r="J86" s="51" t="n"/>
+      <c r="K86" s="51" t="n"/>
+    </row>
+    <row r="87" ht="18.75" customHeight="1">
+      <c r="B87" s="58" t="n"/>
+      <c r="C87" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_DIA@@</t>
+        </is>
+      </c>
+      <c r="D87" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_MES@@</t>
+        </is>
+      </c>
+      <c r="E87" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_ANIO@@</t>
+        </is>
+      </c>
+      <c r="F87" s="51" t="n"/>
+      <c r="G87" s="51" t="n"/>
+      <c r="H87" s="51" t="n"/>
+      <c r="I87" s="51" t="n"/>
+      <c r="J87" s="51" t="n"/>
+      <c r="K87" s="51" t="n"/>
+    </row>
+    <row r="88" ht="18.75" customHeight="1">
+      <c r="B88" s="52" t="inlineStr">
+        <is>
+          <t>FECHA REVISIÓN:</t>
+        </is>
+      </c>
+      <c r="C88" s="57" t="n"/>
+      <c r="D88" s="57" t="n"/>
+      <c r="E88" s="53" t="n"/>
+      <c r="F88" s="51" t="n"/>
+      <c r="G88" s="51" t="n"/>
+      <c r="H88" s="51" t="n"/>
+      <c r="I88" s="51" t="n"/>
+      <c r="J88" s="51" t="n"/>
+      <c r="K88" s="51" t="n"/>
+    </row>
+    <row r="89" ht="18.75" customHeight="1">
+      <c r="B89" s="52" t="inlineStr">
+        <is>
+          <t>REVISADO  POR:</t>
+        </is>
+      </c>
+      <c r="C89" s="302" t="inlineStr">
+        <is>
+          <t>@@REVISADO_POR@@</t>
+        </is>
+      </c>
+      <c r="D89" s="275" t="n"/>
+      <c r="E89" s="270" t="n"/>
+      <c r="F89" s="173" t="inlineStr">
+        <is>
+          <t>FIRMA (JEFE DEPARTAMENTO)</t>
+        </is>
+      </c>
+      <c r="H89" s="51" t="n"/>
+      <c r="I89" s="51" t="n"/>
+      <c r="J89" s="51" t="n"/>
+      <c r="K89" s="51" t="n"/>
+    </row>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94" ht="18.75" customHeight="1">
+      <c r="B94" s="169" t="inlineStr">
         <is>
           <t>@@NOTA_PERMISO_CIRCULACION@@</t>
         </is>
       </c>
     </row>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
   </sheetData>
-  <mergeCells count="86">
+  <mergeCells count="98">
     <mergeCell ref="Q21:R21"/>
     <mergeCell ref="C9:S10"/>
     <mergeCell ref="B12:B13"/>
     <mergeCell ref="C30:P30"/>
+    <mergeCell ref="F68:P68"/>
+    <mergeCell ref="B94:K94"/>
     <mergeCell ref="C41:D41"/>
-    <mergeCell ref="F59:P59"/>
     <mergeCell ref="B15:B16"/>
+    <mergeCell ref="F70:P70"/>
+    <mergeCell ref="C43:D43"/>
     <mergeCell ref="G42:P42"/>
     <mergeCell ref="D15:D16"/>
     <mergeCell ref="G8:J8"/>
-    <mergeCell ref="F81:G81"/>
     <mergeCell ref="L25:P25"/>
+    <mergeCell ref="F72:P72"/>
+    <mergeCell ref="E58:P58"/>
+    <mergeCell ref="C77:E77"/>
     <mergeCell ref="C23:P23"/>
-    <mergeCell ref="F56:P56"/>
     <mergeCell ref="E50:P50"/>
+    <mergeCell ref="B37:B44"/>
+    <mergeCell ref="F71:P71"/>
     <mergeCell ref="G37:P37"/>
-    <mergeCell ref="F58:P58"/>
+    <mergeCell ref="C4:S5"/>
     <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="C4:S5"/>
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="E52:P52"/>
-    <mergeCell ref="F60:P60"/>
-    <mergeCell ref="E44:P44"/>
     <mergeCell ref="J15:L15"/>
-    <mergeCell ref="F57:P57"/>
     <mergeCell ref="D27:F27"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="F54:P54"/>
     <mergeCell ref="F63:P63"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="E59:P59"/>
     <mergeCell ref="G41:P41"/>
     <mergeCell ref="E38:F38"/>
     <mergeCell ref="E46:P46"/>
+    <mergeCell ref="L24:P24"/>
     <mergeCell ref="C29:P29"/>
     <mergeCell ref="H27:J27"/>
-    <mergeCell ref="C70:E70"/>
-    <mergeCell ref="L24:P24"/>
     <mergeCell ref="C40:D40"/>
+    <mergeCell ref="G43:P43"/>
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="D25:F25"/>
     <mergeCell ref="L8:P8"/>
-    <mergeCell ref="C81:E81"/>
-    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="E57:P57"/>
+    <mergeCell ref="E54:P54"/>
+    <mergeCell ref="B47:B60"/>
     <mergeCell ref="F62:P62"/>
     <mergeCell ref="E47:P47"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="F61:P61"/>
+    <mergeCell ref="E56:P56"/>
+    <mergeCell ref="C89:E89"/>
     <mergeCell ref="B7:S7"/>
     <mergeCell ref="M15:S15"/>
-    <mergeCell ref="B45:B52"/>
     <mergeCell ref="F64:P64"/>
+    <mergeCell ref="E60:P60"/>
+    <mergeCell ref="F89:G89"/>
     <mergeCell ref="E39:F39"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="G44:P44"/>
     <mergeCell ref="G40:P40"/>
     <mergeCell ref="Q20:R20"/>
-    <mergeCell ref="E45:P45"/>
     <mergeCell ref="E15:E16"/>
+    <mergeCell ref="C44:D44"/>
     <mergeCell ref="G15:G16"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="H24:J24"/>
-    <mergeCell ref="C69:E69"/>
-    <mergeCell ref="B86:K86"/>
+    <mergeCell ref="F66:P66"/>
+    <mergeCell ref="C78:E78"/>
     <mergeCell ref="C38:D38"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="L27:P27"/>
+    <mergeCell ref="E51:P51"/>
+    <mergeCell ref="D28:P28"/>
+    <mergeCell ref="E43:F43"/>
     <mergeCell ref="F15:F16"/>
-    <mergeCell ref="E51:P51"/>
     <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="D28:P28"/>
+    <mergeCell ref="F69:P69"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="E42:F42"/>
+    <mergeCell ref="F65:P65"/>
     <mergeCell ref="C12:S13"/>
     <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="F55:P55"/>
+    <mergeCell ref="C76:E76"/>
+    <mergeCell ref="B75:E75"/>
     <mergeCell ref="E49:P49"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="Q19:R19"/>
     <mergeCell ref="D24:F24"/>
-    <mergeCell ref="B37:B42"/>
     <mergeCell ref="G39:P39"/>
-    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="E53:P53"/>
+    <mergeCell ref="C83:E83"/>
+    <mergeCell ref="C39:D39"/>
     <mergeCell ref="G38:P38"/>
-    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="F67:P67"/>
+    <mergeCell ref="E55:P55"/>
     <mergeCell ref="C37:D37"/>
+    <mergeCell ref="C15:C16"/>
     <mergeCell ref="E37:F37"/>
-    <mergeCell ref="C15:C16"/>
     <mergeCell ref="E48:P48"/>
     <mergeCell ref="H25:J25"/>
   </mergeCells>

</xml_diff>

<commit_message>
Ficha de terreno: viático con hasta 4 profesionales (botón Agregar profesional), filas nuevas en la plantilla; SW v15. Verificado con datos de prueba.
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/plantilla_ficha_terreno.xlsx
+++ b/assets/plantilla_ficha_terreno.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Informe PLANIFICACION" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Informe PLANIFICACION'!$B$1:$P$71</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Informe PLANIFICACION'!$B$1:$P$74</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -2356,7 +2356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:T94"/>
+  <dimension ref="A1:T97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="68.7109375" customWidth="1" min="2" max="2"/>
@@ -3596,7 +3596,7 @@
     <row r="33" ht="24.75" customHeight="1">
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>Profesional</t>
+          <t>@@VIA_P1_LBL@@</t>
         </is>
       </c>
       <c r="C33" s="59" t="inlineStr">
@@ -3635,273 +3635,298 @@
       <c r="S33" s="10" t="n"/>
       <c r="T33" s="10" t="n"/>
     </row>
-    <row r="34" ht="19.5" customHeight="1" thickBot="1">
+    <row r="34" ht="24.75" customHeight="1" thickBot="1">
       <c r="B34" s="17" t="inlineStr">
         <is>
+          <t>@@VIA_P2_LBL@@</t>
+        </is>
+      </c>
+      <c r="C34" s="59" t="inlineStr">
+        <is>
+          <t>@@VIA_P2_C@@</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>@@VIA_P2_D@@</t>
+        </is>
+      </c>
+      <c r="E34" s="278" t="inlineStr">
+        <is>
+          <t>@@VIA_P2_E@@</t>
+        </is>
+      </c>
+      <c r="F34" s="280" t="inlineStr">
+        <is>
+          <t>@@VIA_P2_F@@</t>
+        </is>
+      </c>
+      <c r="G34" s="281" t="inlineStr">
+        <is>
+          <t>@@VIA_P2_G@@</t>
+        </is>
+      </c>
+      <c r="O34" s="282" t="n"/>
+      <c r="P34" s="283" t="n"/>
+      <c r="Q34" s="10" t="n"/>
+      <c r="R34" s="10" t="n"/>
+      <c r="S34" s="10" t="n"/>
+      <c r="T34" s="10" t="n"/>
+    </row>
+    <row r="35" ht="24.75" customHeight="1" thickBot="1">
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_LBL@@</t>
+        </is>
+      </c>
+      <c r="C35" s="59" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_C@@</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_D@@</t>
+        </is>
+      </c>
+      <c r="E35" s="278" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_E@@</t>
+        </is>
+      </c>
+      <c r="F35" s="280" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_F@@</t>
+        </is>
+      </c>
+      <c r="G35" s="281" t="inlineStr">
+        <is>
+          <t>@@VIA_P3_G@@</t>
+        </is>
+      </c>
+      <c r="O35" s="282" t="n"/>
+      <c r="P35" s="283" t="n"/>
+      <c r="Q35" s="10" t="n"/>
+      <c r="R35" s="10" t="n"/>
+      <c r="S35" s="10" t="n"/>
+      <c r="T35" s="10" t="n"/>
+    </row>
+    <row r="36" ht="24.75" customHeight="1" thickBot="1">
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_LBL@@</t>
+        </is>
+      </c>
+      <c r="C36" s="59" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_C@@</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_D@@</t>
+        </is>
+      </c>
+      <c r="E36" s="278" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_E@@</t>
+        </is>
+      </c>
+      <c r="F36" s="280" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_F@@</t>
+        </is>
+      </c>
+      <c r="G36" s="281" t="inlineStr">
+        <is>
+          <t>@@VIA_P4_G@@</t>
+        </is>
+      </c>
+      <c r="O36" s="282" t="n"/>
+      <c r="P36" s="283" t="n"/>
+      <c r="Q36" s="10" t="n"/>
+      <c r="R36" s="10" t="n"/>
+      <c r="S36" s="10" t="n"/>
+      <c r="T36" s="10" t="n"/>
+    </row>
+    <row r="37" ht="19.5" customHeight="1" thickBot="1">
+      <c r="B37" s="17" t="inlineStr">
+        <is>
           <t>Administrativo</t>
         </is>
       </c>
-      <c r="C34" s="28" t="inlineStr">
+      <c r="C37" s="28" t="inlineStr">
         <is>
           <t>@@VIA_C34@@</t>
         </is>
       </c>
-      <c r="D34" s="28" t="inlineStr">
+      <c r="D37" s="28" t="inlineStr">
         <is>
           <t>@@VIA_D34@@</t>
         </is>
       </c>
-      <c r="E34" s="280" t="inlineStr">
+      <c r="E37" s="280" t="inlineStr">
         <is>
           <t>@@VIA_E34@@</t>
         </is>
       </c>
-      <c r="F34" s="280" t="inlineStr">
+      <c r="F37" s="280" t="inlineStr">
         <is>
           <t>@@VIA_F34@@</t>
         </is>
       </c>
-      <c r="G34" s="281" t="inlineStr">
+      <c r="G37" s="281" t="inlineStr">
         <is>
           <t>@@VIA_G34@@</t>
         </is>
       </c>
-      <c r="O34" s="284" t="n">
+      <c r="O37" s="284" t="n">
         <v>58501</v>
       </c>
-      <c r="P34" s="285" t="n">
+      <c r="P37" s="285" t="n">
         <v>23400</v>
       </c>
-      <c r="Q34" s="1" t="n"/>
-      <c r="R34" s="1" t="n"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1" thickBot="1">
-      <c r="B35" s="44" t="inlineStr">
+      <c r="Q37" s="1" t="n"/>
+      <c r="R37" s="1" t="n"/>
+    </row>
+    <row r="38" ht="19.5" customHeight="1">
+      <c r="B38" s="44" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C35" s="45" t="inlineStr">
+      <c r="C38" s="45" t="inlineStr">
         <is>
           <t>@@VIA_C35@@</t>
         </is>
       </c>
-      <c r="D35" s="46" t="inlineStr">
+      <c r="D38" s="46" t="inlineStr">
         <is>
           <t>@@VIA_D35@@</t>
         </is>
       </c>
-      <c r="E35" s="286" t="inlineStr">
+      <c r="E38" s="286" t="inlineStr">
         <is>
           <t>@@VIA_E35@@</t>
         </is>
       </c>
-      <c r="F35" s="286" t="inlineStr">
+      <c r="F38" s="286" t="inlineStr">
         <is>
           <t>@@VIA_F35@@</t>
         </is>
       </c>
-      <c r="G35" s="287" t="inlineStr">
+      <c r="G38" s="287" t="inlineStr">
         <is>
           <t>@@VIA_G35@@</t>
         </is>
       </c>
-      <c r="K35" s="288" t="n"/>
-      <c r="Q35" s="1" t="n"/>
-      <c r="R35" s="1" t="n"/>
-    </row>
-    <row r="36" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B36" s="7" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="197" t="n"/>
-      <c r="E36" s="197" t="n"/>
-      <c r="F36" s="197" t="n"/>
-      <c r="G36" s="197" t="n"/>
-      <c r="H36" s="197" t="n"/>
-      <c r="I36" s="6" t="n"/>
-      <c r="J36" s="6" t="n"/>
-      <c r="K36" s="1" t="n"/>
-      <c r="L36" s="1" t="n"/>
-      <c r="M36" s="1" t="n"/>
-      <c r="N36" s="1" t="n"/>
-      <c r="O36" s="1" t="n"/>
-      <c r="P36" s="1" t="n"/>
-      <c r="Q36" s="4" t="n"/>
-      <c r="R36" s="4" t="n"/>
-    </row>
-    <row r="37" ht="39" customHeight="1" thickBot="1">
-      <c r="B37" s="289" t="inlineStr">
+      <c r="K38" s="288" t="n"/>
+      <c r="Q38" s="1" t="n"/>
+      <c r="R38" s="1" t="n"/>
+    </row>
+    <row r="39" ht="22.5" customHeight="1">
+      <c r="B39" s="7" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="197" t="n"/>
+      <c r="E39" s="197" t="n"/>
+      <c r="F39" s="197" t="n"/>
+      <c r="G39" s="197" t="n"/>
+      <c r="H39" s="197" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="n"/>
+      <c r="K39" s="1" t="n"/>
+      <c r="L39" s="1" t="n"/>
+      <c r="M39" s="1" t="n"/>
+      <c r="N39" s="1" t="n"/>
+      <c r="O39" s="1" t="n"/>
+      <c r="P39" s="1" t="n"/>
+      <c r="Q39" s="4" t="n"/>
+      <c r="R39" s="4" t="n"/>
+    </row>
+    <row r="40" ht="39" customHeight="1">
+      <c r="B40" s="289" t="inlineStr">
         <is>
           <t>Fondos a Rendir
 SOLICITADOS [$]</t>
         </is>
       </c>
-      <c r="C37" s="290" t="inlineStr">
+      <c r="C40" s="290" t="inlineStr">
         <is>
           <t>Conceptos de gastos presupuestados</t>
         </is>
       </c>
-      <c r="D37" s="277" t="n"/>
-      <c r="E37" s="132" t="inlineStr">
+      <c r="D40" s="277" t="n"/>
+      <c r="E40" s="132" t="inlineStr">
         <is>
           <t>MONTO [$]</t>
         </is>
       </c>
-      <c r="F37" s="268" t="n"/>
-      <c r="G37" s="132" t="inlineStr">
+      <c r="F40" s="268" t="n"/>
+      <c r="G40" s="132" t="inlineStr">
         <is>
           <t>DETALLE</t>
         </is>
       </c>
-      <c r="H37" s="84" t="n"/>
-      <c r="I37" s="84" t="n"/>
-      <c r="J37" s="84" t="n"/>
-      <c r="K37" s="84" t="n"/>
-      <c r="L37" s="84" t="n"/>
-      <c r="M37" s="84" t="n"/>
-      <c r="N37" s="84" t="n"/>
-      <c r="O37" s="84" t="n"/>
-      <c r="P37" s="268" t="n"/>
-      <c r="Q37" s="4" t="n"/>
-      <c r="R37" s="4" t="n"/>
-    </row>
-    <row r="38" ht="22.5" customHeight="1">
-      <c r="B38" s="291" t="n"/>
-      <c r="C38" s="153" t="inlineStr">
-        <is>
-          <t>Imprevistos</t>
-        </is>
-      </c>
-      <c r="D38" s="270" t="n"/>
-      <c r="E38" s="278" t="inlineStr">
-        <is>
-          <t>@@FONDOS_E38@@</t>
-        </is>
-      </c>
-      <c r="F38" s="258" t="n"/>
-      <c r="G38" s="195" t="inlineStr">
-        <is>
-          <t>@@FONDOS_DET_G38@@</t>
-        </is>
-      </c>
-      <c r="H38" s="257" t="n"/>
-      <c r="I38" s="257" t="n"/>
-      <c r="J38" s="257" t="n"/>
-      <c r="K38" s="257" t="n"/>
-      <c r="L38" s="257" t="n"/>
-      <c r="M38" s="257" t="n"/>
-      <c r="N38" s="257" t="n"/>
-      <c r="O38" s="257" t="n"/>
-      <c r="P38" s="258" t="n"/>
-      <c r="Q38" s="4" t="n"/>
-      <c r="R38" s="4" t="n"/>
-    </row>
-    <row r="39" ht="22.5" customHeight="1">
-      <c r="B39" s="291" t="n"/>
-      <c r="C39" s="292" t="inlineStr">
-        <is>
-          <t>Lavado de Camioneta</t>
-        </is>
-      </c>
-      <c r="D39" s="270" t="n"/>
-      <c r="E39" s="278" t="inlineStr">
-        <is>
-          <t>@@FONDOS_E39@@</t>
-        </is>
-      </c>
-      <c r="F39" s="258" t="n"/>
-      <c r="G39" s="293" t="inlineStr">
-        <is>
-          <t>@@FONDOS_DET_G39@@</t>
-        </is>
-      </c>
-      <c r="H39" s="275" t="n"/>
-      <c r="I39" s="275" t="n"/>
-      <c r="J39" s="275" t="n"/>
-      <c r="K39" s="275" t="n"/>
-      <c r="L39" s="275" t="n"/>
-      <c r="M39" s="275" t="n"/>
-      <c r="N39" s="275" t="n"/>
-      <c r="O39" s="275" t="n"/>
-      <c r="P39" s="279" t="n"/>
-      <c r="Q39" s="4" t="n"/>
-      <c r="R39" s="4" t="n"/>
-    </row>
-    <row r="40" ht="18.75" customHeight="1">
-      <c r="B40" s="291" t="n"/>
-      <c r="C40" s="153" t="inlineStr">
-        <is>
-          <t>Peajes</t>
-        </is>
-      </c>
-      <c r="D40" s="270" t="n"/>
-      <c r="E40" s="280" t="inlineStr">
-        <is>
-          <t>@@FONDOS_E40@@</t>
-        </is>
-      </c>
-      <c r="F40" s="270" t="n"/>
-      <c r="G40" s="227" t="inlineStr">
-        <is>
-          <t>@@FONDOS_DET_G40@@</t>
-        </is>
-      </c>
-      <c r="H40" s="275" t="n"/>
-      <c r="I40" s="275" t="n"/>
-      <c r="J40" s="275" t="n"/>
-      <c r="K40" s="275" t="n"/>
-      <c r="L40" s="275" t="n"/>
-      <c r="M40" s="275" t="n"/>
-      <c r="N40" s="275" t="n"/>
-      <c r="O40" s="275" t="n"/>
-      <c r="P40" s="270" t="n"/>
-    </row>
-    <row r="41" ht="18.75" customHeight="1" thickBot="1">
+      <c r="H40" s="84" t="n"/>
+      <c r="I40" s="84" t="n"/>
+      <c r="J40" s="84" t="n"/>
+      <c r="K40" s="84" t="n"/>
+      <c r="L40" s="84" t="n"/>
+      <c r="M40" s="84" t="n"/>
+      <c r="N40" s="84" t="n"/>
+      <c r="O40" s="84" t="n"/>
+      <c r="P40" s="268" t="n"/>
+      <c r="Q40" s="4" t="n"/>
+      <c r="R40" s="4" t="n"/>
+    </row>
+    <row r="41" ht="22.5" customHeight="1" thickBot="1">
       <c r="B41" s="291" t="n"/>
       <c r="C41" s="153" t="inlineStr">
         <is>
-          <t>Alarife (líquido)</t>
+          <t>Imprevistos</t>
         </is>
       </c>
       <c r="D41" s="270" t="n"/>
-      <c r="E41" s="280" t="inlineStr">
-        <is>
-          <t>@@FONDOS_ALARIFE@@</t>
-        </is>
-      </c>
-      <c r="F41" s="270" t="n"/>
-      <c r="G41" s="227" t="inlineStr">
-        <is>
-          <t>@@FONDOS_DET_ALARIFE@@</t>
-        </is>
-      </c>
-      <c r="H41" s="275" t="n"/>
-      <c r="I41" s="275" t="n"/>
-      <c r="J41" s="275" t="n"/>
-      <c r="K41" s="275" t="n"/>
-      <c r="L41" s="275" t="n"/>
-      <c r="M41" s="275" t="n"/>
-      <c r="N41" s="275" t="n"/>
-      <c r="O41" s="275" t="n"/>
-      <c r="P41" s="270" t="n"/>
-    </row>
-    <row r="42" ht="18.75" customHeight="1" thickBot="1">
+      <c r="E41" s="278" t="inlineStr">
+        <is>
+          <t>@@FONDOS_E38@@</t>
+        </is>
+      </c>
+      <c r="F41" s="258" t="n"/>
+      <c r="G41" s="195" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_G38@@</t>
+        </is>
+      </c>
+      <c r="H41" s="257" t="n"/>
+      <c r="I41" s="257" t="n"/>
+      <c r="J41" s="257" t="n"/>
+      <c r="K41" s="257" t="n"/>
+      <c r="L41" s="257" t="n"/>
+      <c r="M41" s="257" t="n"/>
+      <c r="N41" s="257" t="n"/>
+      <c r="O41" s="257" t="n"/>
+      <c r="P41" s="258" t="n"/>
+      <c r="Q41" s="4" t="n"/>
+      <c r="R41" s="4" t="n"/>
+    </row>
+    <row r="42" ht="22.5" customHeight="1" thickBot="1">
       <c r="B42" s="291" t="n"/>
-      <c r="C42" s="153" t="inlineStr">
-        <is>
-          <t>Arriendo de caballos (c/ IVA)</t>
+      <c r="C42" s="292" t="inlineStr">
+        <is>
+          <t>Lavado de Camioneta</t>
         </is>
       </c>
       <c r="D42" s="270" t="n"/>
-      <c r="E42" s="280" t="inlineStr">
-        <is>
-          <t>@@FONDOS_CABALLOS@@</t>
-        </is>
-      </c>
-      <c r="F42" s="270" t="n"/>
-      <c r="G42" s="227" t="inlineStr">
-        <is>
-          <t>@@FONDOS_DET_CABALLOS@@</t>
+      <c r="E42" s="278" t="inlineStr">
+        <is>
+          <t>@@FONDOS_E39@@</t>
+        </is>
+      </c>
+      <c r="F42" s="258" t="n"/>
+      <c r="G42" s="293" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_G39@@</t>
         </is>
       </c>
       <c r="H42" s="275" t="n"/>
@@ -3912,240 +3937,242 @@
       <c r="M42" s="275" t="n"/>
       <c r="N42" s="275" t="n"/>
       <c r="O42" s="275" t="n"/>
-      <c r="P42" s="270" t="n"/>
-    </row>
-    <row r="43" ht="21.75" customHeight="1" thickBot="1">
+      <c r="P42" s="279" t="n"/>
+      <c r="Q42" s="4" t="n"/>
+      <c r="R42" s="4" t="n"/>
+    </row>
+    <row r="43" ht="18.75" customHeight="1" thickBot="1">
       <c r="B43" s="291" t="n"/>
-      <c r="C43" s="187" t="inlineStr">
+      <c r="C43" s="153" t="inlineStr">
+        <is>
+          <t>Peajes</t>
+        </is>
+      </c>
+      <c r="D43" s="270" t="n"/>
+      <c r="E43" s="280" t="inlineStr">
+        <is>
+          <t>@@FONDOS_E40@@</t>
+        </is>
+      </c>
+      <c r="F43" s="270" t="n"/>
+      <c r="G43" s="227" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_G40@@</t>
+        </is>
+      </c>
+      <c r="H43" s="275" t="n"/>
+      <c r="I43" s="275" t="n"/>
+      <c r="J43" s="275" t="n"/>
+      <c r="K43" s="275" t="n"/>
+      <c r="L43" s="275" t="n"/>
+      <c r="M43" s="275" t="n"/>
+      <c r="N43" s="275" t="n"/>
+      <c r="O43" s="275" t="n"/>
+      <c r="P43" s="270" t="n"/>
+    </row>
+    <row r="44" ht="18.75" customHeight="1" thickBot="1">
+      <c r="B44" s="291" t="n"/>
+      <c r="C44" s="153" t="inlineStr">
+        <is>
+          <t>Alarife (líquido)</t>
+        </is>
+      </c>
+      <c r="D44" s="270" t="n"/>
+      <c r="E44" s="280" t="inlineStr">
+        <is>
+          <t>@@FONDOS_ALARIFE@@</t>
+        </is>
+      </c>
+      <c r="F44" s="270" t="n"/>
+      <c r="G44" s="227" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_ALARIFE@@</t>
+        </is>
+      </c>
+      <c r="H44" s="275" t="n"/>
+      <c r="I44" s="275" t="n"/>
+      <c r="J44" s="275" t="n"/>
+      <c r="K44" s="275" t="n"/>
+      <c r="L44" s="275" t="n"/>
+      <c r="M44" s="275" t="n"/>
+      <c r="N44" s="275" t="n"/>
+      <c r="O44" s="275" t="n"/>
+      <c r="P44" s="270" t="n"/>
+    </row>
+    <row r="45" ht="18.75" customHeight="1">
+      <c r="B45" s="291" t="n"/>
+      <c r="C45" s="153" t="inlineStr">
+        <is>
+          <t>Arriendo de caballos (c/ IVA)</t>
+        </is>
+      </c>
+      <c r="D45" s="270" t="n"/>
+      <c r="E45" s="280" t="inlineStr">
+        <is>
+          <t>@@FONDOS_CABALLOS@@</t>
+        </is>
+      </c>
+      <c r="F45" s="270" t="n"/>
+      <c r="G45" s="227" t="inlineStr">
+        <is>
+          <t>@@FONDOS_DET_CABALLOS@@</t>
+        </is>
+      </c>
+      <c r="H45" s="275" t="n"/>
+      <c r="I45" s="275" t="n"/>
+      <c r="J45" s="275" t="n"/>
+      <c r="K45" s="275" t="n"/>
+      <c r="L45" s="275" t="n"/>
+      <c r="M45" s="275" t="n"/>
+      <c r="N45" s="275" t="n"/>
+      <c r="O45" s="275" t="n"/>
+      <c r="P45" s="270" t="n"/>
+    </row>
+    <row r="46" ht="21.75" customHeight="1">
+      <c r="B46" s="291" t="n"/>
+      <c r="C46" s="187" t="inlineStr">
         <is>
           <t>@@FONDOS_OTRO_LABEL@@</t>
         </is>
       </c>
-      <c r="D43" s="271" t="n"/>
-      <c r="E43" s="280" t="inlineStr">
+      <c r="D46" s="271" t="n"/>
+      <c r="E46" s="280" t="inlineStr">
         <is>
           <t>@@FONDOS_E41@@</t>
         </is>
       </c>
-      <c r="F43" s="270" t="n"/>
-      <c r="G43" s="231" t="inlineStr">
+      <c r="F46" s="270" t="n"/>
+      <c r="G46" s="231" t="inlineStr">
         <is>
           <t>@@FONDOS_DET_G41@@</t>
         </is>
       </c>
-      <c r="H43" s="276" t="n"/>
-      <c r="I43" s="276" t="n"/>
-      <c r="J43" s="276" t="n"/>
-      <c r="K43" s="276" t="n"/>
-      <c r="L43" s="276" t="n"/>
-      <c r="M43" s="276" t="n"/>
-      <c r="N43" s="276" t="n"/>
-      <c r="O43" s="276" t="n"/>
-      <c r="P43" s="271" t="n"/>
-    </row>
-    <row r="44" ht="22.5" customHeight="1" thickBot="1">
-      <c r="B44" s="294" t="n"/>
-      <c r="C44" s="200" t="inlineStr">
+      <c r="H46" s="276" t="n"/>
+      <c r="I46" s="276" t="n"/>
+      <c r="J46" s="276" t="n"/>
+      <c r="K46" s="276" t="n"/>
+      <c r="L46" s="276" t="n"/>
+      <c r="M46" s="276" t="n"/>
+      <c r="N46" s="276" t="n"/>
+      <c r="O46" s="276" t="n"/>
+      <c r="P46" s="271" t="n"/>
+    </row>
+    <row r="47" ht="22.5" customHeight="1">
+      <c r="B47" s="294" t="n"/>
+      <c r="C47" s="200" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D44" s="295" t="n"/>
-      <c r="E44" s="296" t="inlineStr">
+      <c r="D47" s="295" t="n"/>
+      <c r="E47" s="296" t="inlineStr">
         <is>
           <t>@@FONDOS_E42@@</t>
         </is>
       </c>
-      <c r="F44" s="253" t="n"/>
-      <c r="G44" s="197" t="n"/>
-      <c r="Q44" s="13" t="n"/>
-      <c r="R44" s="13" t="n"/>
-    </row>
-    <row r="45" ht="22.5" customHeight="1">
-      <c r="B45" s="7" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="197" t="n"/>
-      <c r="F45" s="197" t="n"/>
-      <c r="G45" s="197" t="n"/>
-      <c r="H45" s="197" t="n"/>
-      <c r="I45" s="197" t="n"/>
-      <c r="J45" s="197" t="n"/>
-      <c r="K45" s="197" t="n"/>
-      <c r="L45" s="197" t="n"/>
-      <c r="M45" s="197" t="n"/>
-      <c r="N45" s="197" t="n"/>
-      <c r="Q45" s="13" t="n"/>
-      <c r="R45" s="13" t="n"/>
-    </row>
-    <row r="46" ht="22.5" customHeight="1">
-      <c r="B46" s="104" t="inlineStr">
-        <is>
-          <t>ACTIVIDADES / OBJETIVOS</t>
-        </is>
-      </c>
-      <c r="C46" s="229" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="D46" s="106" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> # DIAS</t>
-        </is>
-      </c>
-      <c r="E46" s="229" t="inlineStr">
-        <is>
-          <t>ACTIVIDAD / OBJETIVO</t>
-        </is>
-      </c>
-      <c r="F46" s="84" t="n"/>
-      <c r="G46" s="84" t="n"/>
-      <c r="H46" s="84" t="n"/>
-      <c r="I46" s="84" t="n"/>
-      <c r="J46" s="84" t="n"/>
-      <c r="K46" s="84" t="n"/>
-      <c r="L46" s="84" t="n"/>
-      <c r="M46" s="84" t="n"/>
-      <c r="N46" s="84" t="n"/>
-      <c r="O46" s="84" t="n"/>
-      <c r="P46" s="268" t="n"/>
-      <c r="Q46" s="13" t="n"/>
-      <c r="R46" s="13" t="n"/>
-    </row>
-    <row r="47" ht="22.5" customHeight="1">
-      <c r="B47" s="181" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Detalle de actividades (diarias o por periodos) u objetivos a realizar durante cometido </t>
-        </is>
-      </c>
-      <c r="C47" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="D47" s="103" t="inlineStr">
-        <is>
-          <t>@@ACT1_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E47" s="235" t="inlineStr">
-        <is>
-          <t>@@ACT1_DESC@@</t>
-        </is>
-      </c>
-      <c r="F47" s="257" t="n"/>
-      <c r="G47" s="257" t="n"/>
-      <c r="H47" s="257" t="n"/>
-      <c r="I47" s="257" t="n"/>
-      <c r="J47" s="257" t="n"/>
-      <c r="K47" s="257" t="n"/>
-      <c r="L47" s="257" t="n"/>
-      <c r="M47" s="257" t="n"/>
-      <c r="N47" s="257" t="n"/>
-      <c r="O47" s="257" t="n"/>
-      <c r="P47" s="258" t="n"/>
+      <c r="F47" s="253" t="n"/>
+      <c r="G47" s="197" t="n"/>
       <c r="Q47" s="13" t="n"/>
       <c r="R47" s="13" t="n"/>
     </row>
     <row r="48" ht="22.5" customHeight="1">
-      <c r="B48" s="297" t="n"/>
-      <c r="C48" s="141" t="n">
-        <v>2</v>
-      </c>
-      <c r="D48" s="21" t="inlineStr">
-        <is>
-          <t>@@ACT2_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E48" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT2_DESC@@</t>
-        </is>
-      </c>
-      <c r="F48" s="275" t="n"/>
-      <c r="G48" s="275" t="n"/>
-      <c r="H48" s="275" t="n"/>
-      <c r="I48" s="275" t="n"/>
-      <c r="J48" s="275" t="n"/>
-      <c r="K48" s="275" t="n"/>
-      <c r="L48" s="275" t="n"/>
-      <c r="M48" s="275" t="n"/>
-      <c r="N48" s="275" t="n"/>
-      <c r="O48" s="275" t="n"/>
-      <c r="P48" s="270" t="n"/>
+      <c r="B48" s="7" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+      <c r="E48" s="197" t="n"/>
+      <c r="F48" s="197" t="n"/>
+      <c r="G48" s="197" t="n"/>
+      <c r="H48" s="197" t="n"/>
+      <c r="I48" s="197" t="n"/>
+      <c r="J48" s="197" t="n"/>
+      <c r="K48" s="197" t="n"/>
+      <c r="L48" s="197" t="n"/>
+      <c r="M48" s="197" t="n"/>
+      <c r="N48" s="197" t="n"/>
       <c r="Q48" s="13" t="n"/>
       <c r="R48" s="13" t="n"/>
     </row>
     <row r="49" ht="22.5" customHeight="1">
-      <c r="B49" s="297" t="n"/>
-      <c r="C49" s="141" t="n">
-        <v>3</v>
-      </c>
-      <c r="D49" s="21" t="inlineStr">
-        <is>
-          <t>@@ACT3_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E49" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT3_DESC@@</t>
-        </is>
-      </c>
-      <c r="F49" s="275" t="n"/>
-      <c r="G49" s="275" t="n"/>
-      <c r="H49" s="275" t="n"/>
-      <c r="I49" s="275" t="n"/>
-      <c r="J49" s="275" t="n"/>
-      <c r="K49" s="275" t="n"/>
-      <c r="L49" s="275" t="n"/>
-      <c r="M49" s="275" t="n"/>
-      <c r="N49" s="275" t="n"/>
-      <c r="O49" s="275" t="n"/>
-      <c r="P49" s="270" t="n"/>
+      <c r="B49" s="104" t="inlineStr">
+        <is>
+          <t>ACTIVIDADES / OBJETIVOS</t>
+        </is>
+      </c>
+      <c r="C49" s="229" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="D49" s="106" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> # DIAS</t>
+        </is>
+      </c>
+      <c r="E49" s="229" t="inlineStr">
+        <is>
+          <t>ACTIVIDAD / OBJETIVO</t>
+        </is>
+      </c>
+      <c r="F49" s="84" t="n"/>
+      <c r="G49" s="84" t="n"/>
+      <c r="H49" s="84" t="n"/>
+      <c r="I49" s="84" t="n"/>
+      <c r="J49" s="84" t="n"/>
+      <c r="K49" s="84" t="n"/>
+      <c r="L49" s="84" t="n"/>
+      <c r="M49" s="84" t="n"/>
+      <c r="N49" s="84" t="n"/>
+      <c r="O49" s="84" t="n"/>
+      <c r="P49" s="268" t="n"/>
       <c r="Q49" s="13" t="n"/>
       <c r="R49" s="13" t="n"/>
     </row>
     <row r="50" ht="22.5" customHeight="1">
-      <c r="B50" s="297" t="n"/>
-      <c r="C50" s="141" t="n">
-        <v>4</v>
-      </c>
-      <c r="D50" s="21" t="inlineStr">
-        <is>
-          <t>@@ACT4_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E50" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT4_DESC@@</t>
-        </is>
-      </c>
-      <c r="F50" s="275" t="n"/>
-      <c r="G50" s="275" t="n"/>
-      <c r="H50" s="275" t="n"/>
-      <c r="I50" s="275" t="n"/>
-      <c r="J50" s="275" t="n"/>
-      <c r="K50" s="275" t="n"/>
-      <c r="L50" s="275" t="n"/>
-      <c r="M50" s="275" t="n"/>
-      <c r="N50" s="275" t="n"/>
-      <c r="O50" s="275" t="n"/>
-      <c r="P50" s="270" t="n"/>
+      <c r="B50" s="181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Detalle de actividades (diarias o por periodos) u objetivos a realizar durante cometido </t>
+        </is>
+      </c>
+      <c r="C50" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="103" t="inlineStr">
+        <is>
+          <t>@@ACT1_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E50" s="235" t="inlineStr">
+        <is>
+          <t>@@ACT1_DESC@@</t>
+        </is>
+      </c>
+      <c r="F50" s="257" t="n"/>
+      <c r="G50" s="257" t="n"/>
+      <c r="H50" s="257" t="n"/>
+      <c r="I50" s="257" t="n"/>
+      <c r="J50" s="257" t="n"/>
+      <c r="K50" s="257" t="n"/>
+      <c r="L50" s="257" t="n"/>
+      <c r="M50" s="257" t="n"/>
+      <c r="N50" s="257" t="n"/>
+      <c r="O50" s="257" t="n"/>
+      <c r="P50" s="258" t="n"/>
       <c r="Q50" s="13" t="n"/>
       <c r="R50" s="13" t="n"/>
     </row>
     <row r="51" ht="22.5" customHeight="1">
       <c r="B51" s="297" t="n"/>
       <c r="C51" s="141" t="n">
-        <v>5</v>
-      </c>
-      <c r="D51" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT5_DIAS@@</t>
+        <v>2</v>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>@@ACT2_DIAS@@</t>
         </is>
       </c>
       <c r="E51" s="151" t="inlineStr">
         <is>
-          <t>@@ACT5_DESC@@</t>
+          <t>@@ACT2_DESC@@</t>
         </is>
       </c>
       <c r="F51" s="275" t="n"/>
@@ -4162,19 +4189,19 @@
       <c r="Q51" s="13" t="n"/>
       <c r="R51" s="13" t="n"/>
     </row>
-    <row r="52" ht="18.75" customHeight="1" thickBot="1">
+    <row r="52" ht="22.5" customHeight="1" thickBot="1">
       <c r="B52" s="297" t="n"/>
       <c r="C52" s="141" t="n">
-        <v>6</v>
-      </c>
-      <c r="D52" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT6_DIAS@@</t>
+        <v>3</v>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>@@ACT3_DIAS@@</t>
         </is>
       </c>
       <c r="E52" s="151" t="inlineStr">
         <is>
-          <t>@@ACT6_DESC@@</t>
+          <t>@@ACT3_DESC@@</t>
         </is>
       </c>
       <c r="F52" s="275" t="n"/>
@@ -4188,23 +4215,22 @@
       <c r="N52" s="275" t="n"/>
       <c r="O52" s="275" t="n"/>
       <c r="P52" s="270" t="n"/>
-      <c r="Q52" s="1" t="n"/>
-      <c r="R52" s="1" t="n"/>
-    </row>
-    <row r="53" ht="18.75" customHeight="1" thickBot="1">
-      <c r="A53" s="1" t="n"/>
+      <c r="Q52" s="13" t="n"/>
+      <c r="R52" s="13" t="n"/>
+    </row>
+    <row r="53" ht="22.5" customHeight="1" thickBot="1">
       <c r="B53" s="297" t="n"/>
       <c r="C53" s="141" t="n">
-        <v>7</v>
-      </c>
-      <c r="D53" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT7_DIAS@@</t>
+        <v>4</v>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>@@ACT4_DIAS@@</t>
         </is>
       </c>
       <c r="E53" s="151" t="inlineStr">
         <is>
-          <t>@@ACT7_DESC@@</t>
+          <t>@@ACT4_DESC@@</t>
         </is>
       </c>
       <c r="F53" s="275" t="n"/>
@@ -4218,49 +4244,51 @@
       <c r="N53" s="275" t="n"/>
       <c r="O53" s="275" t="n"/>
       <c r="P53" s="270" t="n"/>
-    </row>
-    <row r="54" ht="24" customHeight="1" thickBot="1">
-      <c r="A54" s="1" t="n"/>
+      <c r="Q53" s="13" t="n"/>
+      <c r="R53" s="13" t="n"/>
+    </row>
+    <row r="54" ht="22.5" customHeight="1" thickBot="1">
       <c r="B54" s="297" t="n"/>
-      <c r="C54" s="139" t="n">
-        <v>8</v>
-      </c>
-      <c r="D54" s="30" t="inlineStr">
-        <is>
-          <t>@@ACT8_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E54" s="198" t="inlineStr">
-        <is>
-          <t>@@ACT8_DESC@@</t>
-        </is>
-      </c>
-      <c r="F54" s="276" t="n"/>
-      <c r="G54" s="276" t="n"/>
-      <c r="H54" s="276" t="n"/>
-      <c r="I54" s="276" t="n"/>
-      <c r="J54" s="276" t="n"/>
-      <c r="K54" s="276" t="n"/>
-      <c r="L54" s="276" t="n"/>
-      <c r="M54" s="276" t="n"/>
-      <c r="N54" s="276" t="n"/>
-      <c r="O54" s="276" t="n"/>
-      <c r="P54" s="271" t="n"/>
+      <c r="C54" s="141" t="n">
+        <v>5</v>
+      </c>
+      <c r="D54" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT5_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E54" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT5_DESC@@</t>
+        </is>
+      </c>
+      <c r="F54" s="275" t="n"/>
+      <c r="G54" s="275" t="n"/>
+      <c r="H54" s="275" t="n"/>
+      <c r="I54" s="275" t="n"/>
+      <c r="J54" s="275" t="n"/>
+      <c r="K54" s="275" t="n"/>
+      <c r="L54" s="275" t="n"/>
+      <c r="M54" s="275" t="n"/>
+      <c r="N54" s="275" t="n"/>
+      <c r="O54" s="275" t="n"/>
+      <c r="P54" s="270" t="n"/>
+      <c r="Q54" s="13" t="n"/>
+      <c r="R54" s="13" t="n"/>
     </row>
     <row r="55" ht="18.75" customHeight="1">
-      <c r="A55" s="1" t="n"/>
       <c r="B55" s="297" t="n"/>
       <c r="C55" s="141" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D55" s="22" t="inlineStr">
         <is>
-          <t>@@ACT9_DIAS@@</t>
+          <t>@@ACT6_DIAS@@</t>
         </is>
       </c>
       <c r="E55" s="151" t="inlineStr">
         <is>
-          <t>@@ACT9_DESC@@</t>
+          <t>@@ACT6_DESC@@</t>
         </is>
       </c>
       <c r="F55" s="275" t="n"/>
@@ -4274,21 +4302,23 @@
       <c r="N55" s="275" t="n"/>
       <c r="O55" s="275" t="n"/>
       <c r="P55" s="270" t="n"/>
+      <c r="Q55" s="1" t="n"/>
+      <c r="R55" s="1" t="n"/>
     </row>
     <row r="56" ht="18.75" customHeight="1">
       <c r="A56" s="1" t="n"/>
       <c r="B56" s="297" t="n"/>
       <c r="C56" s="141" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="D56" s="22" t="inlineStr">
         <is>
-          <t>@@ACT10_DIAS@@</t>
+          <t>@@ACT7_DIAS@@</t>
         </is>
       </c>
       <c r="E56" s="151" t="inlineStr">
         <is>
-          <t>@@ACT10_DESC@@</t>
+          <t>@@ACT7_DESC@@</t>
         </is>
       </c>
       <c r="F56" s="275" t="n"/>
@@ -4303,48 +4333,48 @@
       <c r="O56" s="275" t="n"/>
       <c r="P56" s="270" t="n"/>
     </row>
-    <row r="57" ht="18.75" customHeight="1">
+    <row r="57" ht="24" customHeight="1">
       <c r="A57" s="1" t="n"/>
       <c r="B57" s="297" t="n"/>
-      <c r="C57" s="141" t="n">
-        <v>11</v>
-      </c>
-      <c r="D57" s="22" t="inlineStr">
-        <is>
-          <t>@@ACT11_DIAS@@</t>
-        </is>
-      </c>
-      <c r="E57" s="151" t="inlineStr">
-        <is>
-          <t>@@ACT11_DESC@@</t>
-        </is>
-      </c>
-      <c r="F57" s="275" t="n"/>
-      <c r="G57" s="275" t="n"/>
-      <c r="H57" s="275" t="n"/>
-      <c r="I57" s="275" t="n"/>
-      <c r="J57" s="275" t="n"/>
-      <c r="K57" s="275" t="n"/>
-      <c r="L57" s="275" t="n"/>
-      <c r="M57" s="275" t="n"/>
-      <c r="N57" s="275" t="n"/>
-      <c r="O57" s="275" t="n"/>
-      <c r="P57" s="270" t="n"/>
+      <c r="C57" s="139" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" s="30" t="inlineStr">
+        <is>
+          <t>@@ACT8_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E57" s="198" t="inlineStr">
+        <is>
+          <t>@@ACT8_DESC@@</t>
+        </is>
+      </c>
+      <c r="F57" s="276" t="n"/>
+      <c r="G57" s="276" t="n"/>
+      <c r="H57" s="276" t="n"/>
+      <c r="I57" s="276" t="n"/>
+      <c r="J57" s="276" t="n"/>
+      <c r="K57" s="276" t="n"/>
+      <c r="L57" s="276" t="n"/>
+      <c r="M57" s="276" t="n"/>
+      <c r="N57" s="276" t="n"/>
+      <c r="O57" s="276" t="n"/>
+      <c r="P57" s="271" t="n"/>
     </row>
     <row r="58" ht="18.75" customHeight="1">
       <c r="A58" s="1" t="n"/>
       <c r="B58" s="297" t="n"/>
       <c r="C58" s="141" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D58" s="22" t="inlineStr">
         <is>
-          <t>@@ACT12_DIAS@@</t>
+          <t>@@ACT9_DIAS@@</t>
         </is>
       </c>
       <c r="E58" s="151" t="inlineStr">
         <is>
-          <t>@@ACT12_DESC@@</t>
+          <t>@@ACT9_DESC@@</t>
         </is>
       </c>
       <c r="F58" s="275" t="n"/>
@@ -4363,16 +4393,16 @@
       <c r="A59" s="1" t="n"/>
       <c r="B59" s="297" t="n"/>
       <c r="C59" s="141" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D59" s="22" t="inlineStr">
         <is>
-          <t>@@ACT13_DIAS@@</t>
+          <t>@@ACT10_DIAS@@</t>
         </is>
       </c>
       <c r="E59" s="151" t="inlineStr">
         <is>
-          <t>@@ACT13_DESC@@</t>
+          <t>@@ACT10_DESC@@</t>
         </is>
       </c>
       <c r="F59" s="275" t="n"/>
@@ -4389,18 +4419,18 @@
     </row>
     <row r="60" ht="18.75" customHeight="1">
       <c r="A60" s="1" t="n"/>
-      <c r="B60" s="88" t="n"/>
+      <c r="B60" s="297" t="n"/>
       <c r="C60" s="141" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D60" s="22" t="inlineStr">
         <is>
-          <t>@@ACT14_DIAS@@</t>
+          <t>@@ACT11_DIAS@@</t>
         </is>
       </c>
       <c r="E60" s="151" t="inlineStr">
         <is>
-          <t>@@ACT14_DESC@@</t>
+          <t>@@ACT11_DESC@@</t>
         </is>
       </c>
       <c r="F60" s="275" t="n"/>
@@ -4415,238 +4445,209 @@
       <c r="O60" s="275" t="n"/>
       <c r="P60" s="270" t="n"/>
     </row>
-    <row r="61" ht="24" customHeight="1">
+    <row r="61" ht="18.75" customHeight="1">
       <c r="A61" s="1" t="n"/>
-      <c r="B61" s="4" t="n"/>
-      <c r="C61" s="1" t="n"/>
-      <c r="D61" s="1" t="n"/>
-      <c r="E61" s="1" t="n"/>
-      <c r="F61" s="1" t="n"/>
-      <c r="G61" s="1" t="n"/>
-      <c r="H61" s="1" t="n"/>
-      <c r="I61" s="1" t="n"/>
-      <c r="J61" s="1" t="n"/>
-      <c r="K61" s="1" t="n"/>
-      <c r="L61" s="1" t="n"/>
-      <c r="M61" s="1" t="n"/>
-      <c r="N61" s="1" t="n"/>
-      <c r="O61" s="1" t="n"/>
-      <c r="P61" s="1" t="n"/>
-    </row>
-    <row r="62" ht="128.25" customHeight="1">
+      <c r="B61" s="297" t="n"/>
+      <c r="C61" s="141" t="n">
+        <v>12</v>
+      </c>
+      <c r="D61" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT12_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E61" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT12_DESC@@</t>
+        </is>
+      </c>
+      <c r="F61" s="275" t="n"/>
+      <c r="G61" s="275" t="n"/>
+      <c r="H61" s="275" t="n"/>
+      <c r="I61" s="275" t="n"/>
+      <c r="J61" s="275" t="n"/>
+      <c r="K61" s="275" t="n"/>
+      <c r="L61" s="275" t="n"/>
+      <c r="M61" s="275" t="n"/>
+      <c r="N61" s="275" t="n"/>
+      <c r="O61" s="275" t="n"/>
+      <c r="P61" s="270" t="n"/>
+    </row>
+    <row r="62" ht="18.75" customHeight="1">
       <c r="A62" s="1" t="n"/>
-      <c r="B62" s="108" t="inlineStr">
-        <is>
-          <t>Nombre Funcionario</t>
-        </is>
-      </c>
-      <c r="C62" s="109" t="inlineStr">
-        <is>
-          <t>Elementos de Protección Personal asignado</t>
-        </is>
-      </c>
-      <c r="D62" s="110" t="inlineStr">
-        <is>
-          <t>Cantidad</t>
-        </is>
-      </c>
-      <c r="E62" s="229" t="inlineStr">
-        <is>
-          <t>Estado del EPP</t>
-        </is>
-      </c>
-      <c r="F62" s="218" t="inlineStr">
-        <is>
-          <t>Observaciones</t>
-        </is>
-      </c>
-      <c r="G62" s="84" t="n"/>
-      <c r="H62" s="84" t="n"/>
-      <c r="I62" s="84" t="n"/>
-      <c r="J62" s="84" t="n"/>
-      <c r="K62" s="84" t="n"/>
-      <c r="L62" s="84" t="n"/>
-      <c r="M62" s="84" t="n"/>
-      <c r="N62" s="84" t="n"/>
-      <c r="O62" s="84" t="n"/>
-      <c r="P62" s="253" t="n"/>
+      <c r="B62" s="297" t="n"/>
+      <c r="C62" s="141" t="n">
+        <v>13</v>
+      </c>
+      <c r="D62" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT13_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E62" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT13_DESC@@</t>
+        </is>
+      </c>
+      <c r="F62" s="275" t="n"/>
+      <c r="G62" s="275" t="n"/>
+      <c r="H62" s="275" t="n"/>
+      <c r="I62" s="275" t="n"/>
+      <c r="J62" s="275" t="n"/>
+      <c r="K62" s="275" t="n"/>
+      <c r="L62" s="275" t="n"/>
+      <c r="M62" s="275" t="n"/>
+      <c r="N62" s="275" t="n"/>
+      <c r="O62" s="275" t="n"/>
+      <c r="P62" s="270" t="n"/>
     </row>
     <row r="63" ht="18.75" customHeight="1">
       <c r="A63" s="1" t="n"/>
-      <c r="B63" s="107" t="inlineStr">
-        <is>
-          <t>@@EPP1_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C63" s="71" t="inlineStr">
-        <is>
-          <t>@@EPP1_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D63" s="103" t="inlineStr">
-        <is>
-          <t>@@EPP1_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E63" s="103" t="inlineStr">
-        <is>
-          <t>@@EPP1_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F63" s="298" t="inlineStr">
-        <is>
-          <t>@@EPP1_OBS@@</t>
-        </is>
-      </c>
-      <c r="G63" s="257" t="n"/>
-      <c r="H63" s="257" t="n"/>
-      <c r="I63" s="257" t="n"/>
-      <c r="J63" s="257" t="n"/>
-      <c r="K63" s="257" t="n"/>
-      <c r="L63" s="257" t="n"/>
-      <c r="M63" s="257" t="n"/>
-      <c r="N63" s="257" t="n"/>
-      <c r="O63" s="257" t="n"/>
-      <c r="P63" s="299" t="n"/>
-    </row>
-    <row r="64" ht="18.75" customHeight="1" thickBot="1">
+      <c r="B63" s="88" t="n"/>
+      <c r="C63" s="141" t="n">
+        <v>14</v>
+      </c>
+      <c r="D63" s="22" t="inlineStr">
+        <is>
+          <t>@@ACT14_DIAS@@</t>
+        </is>
+      </c>
+      <c r="E63" s="151" t="inlineStr">
+        <is>
+          <t>@@ACT14_DESC@@</t>
+        </is>
+      </c>
+      <c r="F63" s="275" t="n"/>
+      <c r="G63" s="275" t="n"/>
+      <c r="H63" s="275" t="n"/>
+      <c r="I63" s="275" t="n"/>
+      <c r="J63" s="275" t="n"/>
+      <c r="K63" s="275" t="n"/>
+      <c r="L63" s="275" t="n"/>
+      <c r="M63" s="275" t="n"/>
+      <c r="N63" s="275" t="n"/>
+      <c r="O63" s="275" t="n"/>
+      <c r="P63" s="270" t="n"/>
+    </row>
+    <row r="64" ht="24" customHeight="1" thickBot="1">
       <c r="A64" s="1" t="n"/>
-      <c r="B64" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP2_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C64" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP2_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP2_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E64" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP2_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F64" s="166" t="inlineStr">
-        <is>
-          <t>@@EPP2_OBS@@</t>
-        </is>
-      </c>
-      <c r="G64" s="275" t="n"/>
-      <c r="H64" s="275" t="n"/>
-      <c r="I64" s="275" t="n"/>
-      <c r="J64" s="275" t="n"/>
-      <c r="K64" s="275" t="n"/>
-      <c r="L64" s="275" t="n"/>
-      <c r="M64" s="275" t="n"/>
-      <c r="N64" s="275" t="n"/>
-      <c r="O64" s="275" t="n"/>
-      <c r="P64" s="279" t="n"/>
-    </row>
-    <row r="65" ht="18.75" customHeight="1">
+      <c r="B64" s="4" t="n"/>
+      <c r="C64" s="1" t="n"/>
+      <c r="D64" s="1" t="n"/>
+      <c r="E64" s="1" t="n"/>
+      <c r="F64" s="1" t="n"/>
+      <c r="G64" s="1" t="n"/>
+      <c r="H64" s="1" t="n"/>
+      <c r="I64" s="1" t="n"/>
+      <c r="J64" s="1" t="n"/>
+      <c r="K64" s="1" t="n"/>
+      <c r="L64" s="1" t="n"/>
+      <c r="M64" s="1" t="n"/>
+      <c r="N64" s="1" t="n"/>
+      <c r="O64" s="1" t="n"/>
+      <c r="P64" s="1" t="n"/>
+    </row>
+    <row r="65" ht="128.25" customHeight="1">
       <c r="A65" s="1" t="n"/>
-      <c r="B65" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP3_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C65" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP3_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP3_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E65" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP3_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F65" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP3_OBS@@</t>
-        </is>
-      </c>
-      <c r="G65" s="275" t="n"/>
-      <c r="H65" s="275" t="n"/>
-      <c r="I65" s="275" t="n"/>
-      <c r="J65" s="275" t="n"/>
-      <c r="K65" s="275" t="n"/>
-      <c r="L65" s="275" t="n"/>
-      <c r="M65" s="275" t="n"/>
-      <c r="N65" s="275" t="n"/>
-      <c r="O65" s="275" t="n"/>
-      <c r="P65" s="270" t="n"/>
+      <c r="B65" s="108" t="inlineStr">
+        <is>
+          <t>Nombre Funcionario</t>
+        </is>
+      </c>
+      <c r="C65" s="109" t="inlineStr">
+        <is>
+          <t>Elementos de Protección Personal asignado</t>
+        </is>
+      </c>
+      <c r="D65" s="110" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="E65" s="229" t="inlineStr">
+        <is>
+          <t>Estado del EPP</t>
+        </is>
+      </c>
+      <c r="F65" s="218" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="G65" s="84" t="n"/>
+      <c r="H65" s="84" t="n"/>
+      <c r="I65" s="84" t="n"/>
+      <c r="J65" s="84" t="n"/>
+      <c r="K65" s="84" t="n"/>
+      <c r="L65" s="84" t="n"/>
+      <c r="M65" s="84" t="n"/>
+      <c r="N65" s="84" t="n"/>
+      <c r="O65" s="84" t="n"/>
+      <c r="P65" s="253" t="n"/>
     </row>
     <row r="66" ht="18.75" customHeight="1" thickBot="1">
       <c r="A66" s="1" t="n"/>
-      <c r="B66" s="24" t="inlineStr">
-        <is>
-          <t>@@EPP4_NOMBRE@@</t>
-        </is>
-      </c>
-      <c r="C66" s="141" t="inlineStr">
-        <is>
-          <t>@@EPP4_ELEMENTO@@</t>
-        </is>
-      </c>
-      <c r="D66" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP4_CANTIDAD@@</t>
-        </is>
-      </c>
-      <c r="E66" s="21" t="inlineStr">
-        <is>
-          <t>@@EPP4_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F66" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP4_OBS@@</t>
-        </is>
-      </c>
-      <c r="G66" s="275" t="n"/>
-      <c r="H66" s="275" t="n"/>
-      <c r="I66" s="275" t="n"/>
-      <c r="J66" s="275" t="n"/>
-      <c r="K66" s="275" t="n"/>
-      <c r="L66" s="275" t="n"/>
-      <c r="M66" s="275" t="n"/>
-      <c r="N66" s="275" t="n"/>
-      <c r="O66" s="275" t="n"/>
-      <c r="P66" s="270" t="n"/>
+      <c r="B66" s="107" t="inlineStr">
+        <is>
+          <t>@@EPP1_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C66" s="71" t="inlineStr">
+        <is>
+          <t>@@EPP1_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D66" s="103" t="inlineStr">
+        <is>
+          <t>@@EPP1_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E66" s="103" t="inlineStr">
+        <is>
+          <t>@@EPP1_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F66" s="298" t="inlineStr">
+        <is>
+          <t>@@EPP1_OBS@@</t>
+        </is>
+      </c>
+      <c r="G66" s="257" t="n"/>
+      <c r="H66" s="257" t="n"/>
+      <c r="I66" s="257" t="n"/>
+      <c r="J66" s="257" t="n"/>
+      <c r="K66" s="257" t="n"/>
+      <c r="L66" s="257" t="n"/>
+      <c r="M66" s="257" t="n"/>
+      <c r="N66" s="257" t="n"/>
+      <c r="O66" s="257" t="n"/>
+      <c r="P66" s="299" t="n"/>
     </row>
     <row r="67" ht="18.75" customHeight="1">
+      <c r="A67" s="1" t="n"/>
       <c r="B67" s="24" t="inlineStr">
         <is>
-          <t>@@EPP5_NOMBRE@@</t>
+          <t>@@EPP2_NOMBRE@@</t>
         </is>
       </c>
       <c r="C67" s="141" t="inlineStr">
         <is>
-          <t>@@EPP5_ELEMENTO@@</t>
+          <t>@@EPP2_ELEMENTO@@</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
         <is>
-          <t>@@EPP5_CANTIDAD@@</t>
+          <t>@@EPP2_CANTIDAD@@</t>
         </is>
       </c>
       <c r="E67" s="21" t="inlineStr">
         <is>
-          <t>@@EPP5_ESTADO@@</t>
-        </is>
-      </c>
-      <c r="F67" s="165" t="inlineStr">
-        <is>
-          <t>@@EPP5_OBS@@</t>
+          <t>@@EPP2_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F67" s="166" t="inlineStr">
+        <is>
+          <t>@@EPP2_OBS@@</t>
         </is>
       </c>
       <c r="G67" s="275" t="n"/>
@@ -4658,32 +4659,33 @@
       <c r="M67" s="275" t="n"/>
       <c r="N67" s="275" t="n"/>
       <c r="O67" s="275" t="n"/>
-      <c r="P67" s="270" t="n"/>
+      <c r="P67" s="279" t="n"/>
     </row>
     <row r="68" ht="18.75" customHeight="1">
+      <c r="A68" s="1" t="n"/>
       <c r="B68" s="24" t="inlineStr">
         <is>
-          <t>@@EPP6_NOMBRE@@</t>
+          <t>@@EPP3_NOMBRE@@</t>
         </is>
       </c>
       <c r="C68" s="141" t="inlineStr">
         <is>
-          <t>@@EPP6_ELEMENTO@@</t>
+          <t>@@EPP3_ELEMENTO@@</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
         <is>
-          <t>@@EPP6_CANTIDAD@@</t>
+          <t>@@EPP3_CANTIDAD@@</t>
         </is>
       </c>
       <c r="E68" s="21" t="inlineStr">
         <is>
-          <t>@@EPP6_ESTADO@@</t>
+          <t>@@EPP3_ESTADO@@</t>
         </is>
       </c>
       <c r="F68" s="165" t="inlineStr">
         <is>
-          <t>@@EPP6_OBS@@</t>
+          <t>@@EPP3_OBS@@</t>
         </is>
       </c>
       <c r="G68" s="275" t="n"/>
@@ -4698,29 +4700,30 @@
       <c r="P68" s="270" t="n"/>
     </row>
     <row r="69" ht="18.75" customHeight="1">
+      <c r="A69" s="1" t="n"/>
       <c r="B69" s="24" t="inlineStr">
         <is>
-          <t>@@EPP7_NOMBRE@@</t>
+          <t>@@EPP4_NOMBRE@@</t>
         </is>
       </c>
       <c r="C69" s="141" t="inlineStr">
         <is>
-          <t>@@EPP7_ELEMENTO@@</t>
+          <t>@@EPP4_ELEMENTO@@</t>
         </is>
       </c>
       <c r="D69" s="21" t="inlineStr">
         <is>
-          <t>@@EPP7_CANTIDAD@@</t>
+          <t>@@EPP4_CANTIDAD@@</t>
         </is>
       </c>
       <c r="E69" s="21" t="inlineStr">
         <is>
-          <t>@@EPP7_ESTADO@@</t>
+          <t>@@EPP4_ESTADO@@</t>
         </is>
       </c>
       <c r="F69" s="165" t="inlineStr">
         <is>
-          <t>@@EPP7_OBS@@</t>
+          <t>@@EPP4_OBS@@</t>
         </is>
       </c>
       <c r="G69" s="275" t="n"/>
@@ -4737,27 +4740,27 @@
     <row r="70" ht="18.75" customHeight="1" thickBot="1">
       <c r="B70" s="24" t="inlineStr">
         <is>
-          <t>@@EPP8_NOMBRE@@</t>
+          <t>@@EPP5_NOMBRE@@</t>
         </is>
       </c>
       <c r="C70" s="141" t="inlineStr">
         <is>
-          <t>@@EPP8_ELEMENTO@@</t>
+          <t>@@EPP5_ELEMENTO@@</t>
         </is>
       </c>
       <c r="D70" s="21" t="inlineStr">
         <is>
-          <t>@@EPP8_CANTIDAD@@</t>
+          <t>@@EPP5_CANTIDAD@@</t>
         </is>
       </c>
       <c r="E70" s="21" t="inlineStr">
         <is>
-          <t>@@EPP8_ESTADO@@</t>
+          <t>@@EPP5_ESTADO@@</t>
         </is>
       </c>
       <c r="F70" s="165" t="inlineStr">
         <is>
-          <t>@@EPP8_OBS@@</t>
+          <t>@@EPP5_OBS@@</t>
         </is>
       </c>
       <c r="G70" s="275" t="n"/>
@@ -4774,27 +4777,27 @@
     <row r="71" ht="18.75" customHeight="1">
       <c r="B71" s="24" t="inlineStr">
         <is>
-          <t>@@EPP9_NOMBRE@@</t>
+          <t>@@EPP6_NOMBRE@@</t>
         </is>
       </c>
       <c r="C71" s="141" t="inlineStr">
         <is>
-          <t>@@EPP9_ELEMENTO@@</t>
+          <t>@@EPP6_ELEMENTO@@</t>
         </is>
       </c>
       <c r="D71" s="21" t="inlineStr">
         <is>
-          <t>@@EPP9_CANTIDAD@@</t>
+          <t>@@EPP6_CANTIDAD@@</t>
         </is>
       </c>
       <c r="E71" s="21" t="inlineStr">
         <is>
-          <t>@@EPP9_ESTADO@@</t>
+          <t>@@EPP6_ESTADO@@</t>
         </is>
       </c>
       <c r="F71" s="165" t="inlineStr">
         <is>
-          <t>@@EPP9_OBS@@</t>
+          <t>@@EPP6_OBS@@</t>
         </is>
       </c>
       <c r="G71" s="275" t="n"/>
@@ -4808,179 +4811,227 @@
       <c r="O71" s="275" t="n"/>
       <c r="P71" s="270" t="n"/>
     </row>
-    <row r="72" ht="19.5" customHeight="1">
-      <c r="B72" s="98" t="inlineStr">
+    <row r="72" ht="18.75" customHeight="1">
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP7_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C72" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP7_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP7_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E72" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP7_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F72" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP7_OBS@@</t>
+        </is>
+      </c>
+      <c r="G72" s="275" t="n"/>
+      <c r="H72" s="275" t="n"/>
+      <c r="I72" s="275" t="n"/>
+      <c r="J72" s="275" t="n"/>
+      <c r="K72" s="275" t="n"/>
+      <c r="L72" s="275" t="n"/>
+      <c r="M72" s="275" t="n"/>
+      <c r="N72" s="275" t="n"/>
+      <c r="O72" s="275" t="n"/>
+      <c r="P72" s="270" t="n"/>
+    </row>
+    <row r="73" ht="18.75" customHeight="1">
+      <c r="B73" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP8_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C73" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP8_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D73" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP8_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E73" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP8_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F73" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP8_OBS@@</t>
+        </is>
+      </c>
+      <c r="G73" s="275" t="n"/>
+      <c r="H73" s="275" t="n"/>
+      <c r="I73" s="275" t="n"/>
+      <c r="J73" s="275" t="n"/>
+      <c r="K73" s="275" t="n"/>
+      <c r="L73" s="275" t="n"/>
+      <c r="M73" s="275" t="n"/>
+      <c r="N73" s="275" t="n"/>
+      <c r="O73" s="275" t="n"/>
+      <c r="P73" s="270" t="n"/>
+    </row>
+    <row r="74" ht="18.75" customHeight="1">
+      <c r="B74" s="24" t="inlineStr">
+        <is>
+          <t>@@EPP9_NOMBRE@@</t>
+        </is>
+      </c>
+      <c r="C74" s="141" t="inlineStr">
+        <is>
+          <t>@@EPP9_ELEMENTO@@</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP9_CANTIDAD@@</t>
+        </is>
+      </c>
+      <c r="E74" s="21" t="inlineStr">
+        <is>
+          <t>@@EPP9_ESTADO@@</t>
+        </is>
+      </c>
+      <c r="F74" s="165" t="inlineStr">
+        <is>
+          <t>@@EPP9_OBS@@</t>
+        </is>
+      </c>
+      <c r="G74" s="275" t="n"/>
+      <c r="H74" s="275" t="n"/>
+      <c r="I74" s="275" t="n"/>
+      <c r="J74" s="275" t="n"/>
+      <c r="K74" s="275" t="n"/>
+      <c r="L74" s="275" t="n"/>
+      <c r="M74" s="275" t="n"/>
+      <c r="N74" s="275" t="n"/>
+      <c r="O74" s="275" t="n"/>
+      <c r="P74" s="270" t="n"/>
+    </row>
+    <row r="75" ht="19.5" customHeight="1">
+      <c r="B75" s="98" t="inlineStr">
         <is>
           <t>@@EPP10_NOMBRE@@</t>
         </is>
       </c>
-      <c r="C72" s="139" t="inlineStr">
+      <c r="C75" s="139" t="inlineStr">
         <is>
           <t>@@EPP10_ELEMENTO@@</t>
         </is>
       </c>
-      <c r="D72" s="99" t="inlineStr">
+      <c r="D75" s="99" t="inlineStr">
         <is>
           <t>@@EPP10_CANTIDAD@@</t>
         </is>
       </c>
-      <c r="E72" s="99" t="inlineStr">
+      <c r="E75" s="99" t="inlineStr">
         <is>
           <t>@@EPP10_ESTADO@@</t>
         </is>
       </c>
-      <c r="F72" s="167" t="inlineStr">
+      <c r="F75" s="167" t="inlineStr">
         <is>
           <t>@@EPP10_OBS@@</t>
         </is>
       </c>
-      <c r="G72" s="276" t="n"/>
-      <c r="H72" s="276" t="n"/>
-      <c r="I72" s="276" t="n"/>
-      <c r="J72" s="276" t="n"/>
-      <c r="K72" s="276" t="n"/>
-      <c r="L72" s="276" t="n"/>
-      <c r="M72" s="276" t="n"/>
-      <c r="N72" s="276" t="n"/>
-      <c r="O72" s="276" t="n"/>
-      <c r="P72" s="271" t="n"/>
-    </row>
-    <row r="73"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="18.75" customHeight="1">
-      <c r="B75" s="300" t="inlineStr">
+      <c r="G75" s="276" t="n"/>
+      <c r="H75" s="276" t="n"/>
+      <c r="I75" s="276" t="n"/>
+      <c r="J75" s="276" t="n"/>
+      <c r="K75" s="276" t="n"/>
+      <c r="L75" s="276" t="n"/>
+      <c r="M75" s="276" t="n"/>
+      <c r="N75" s="276" t="n"/>
+      <c r="O75" s="276" t="n"/>
+      <c r="P75" s="271" t="n"/>
+    </row>
+    <row r="76"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="18.75" customHeight="1">
+      <c r="B78" s="300" t="inlineStr">
         <is>
           <t>Seguridad y Riesgos</t>
         </is>
       </c>
-      <c r="C75" s="273" t="n"/>
-      <c r="D75" s="273" t="n"/>
-      <c r="E75" s="274" t="n"/>
-    </row>
-    <row r="76" ht="18.75" customHeight="1">
-      <c r="B76" s="17" t="inlineStr">
+      <c r="C78" s="273" t="n"/>
+      <c r="D78" s="273" t="n"/>
+      <c r="E78" s="274" t="n"/>
+    </row>
+    <row r="79" ht="18.75" customHeight="1">
+      <c r="B79" s="17" t="inlineStr">
         <is>
           <t>Identificación de riesgos</t>
         </is>
       </c>
-      <c r="C76" s="166" t="inlineStr">
+      <c r="C79" s="166" t="inlineStr">
         <is>
           <t>@@RIESGOS_IDENT@@</t>
         </is>
       </c>
-      <c r="D76" s="275" t="n"/>
-      <c r="E76" s="279" t="n"/>
-    </row>
-    <row r="77" ht="18.75" customHeight="1">
-      <c r="B77" s="17" t="inlineStr">
+      <c r="D79" s="275" t="n"/>
+      <c r="E79" s="279" t="n"/>
+    </row>
+    <row r="80" ht="18.75" customHeight="1">
+      <c r="B80" s="17" t="inlineStr">
         <is>
           <t>Medidas preventivas</t>
         </is>
       </c>
-      <c r="C77" s="166" t="inlineStr">
+      <c r="C80" s="166" t="inlineStr">
         <is>
           <t>@@RIESGOS_MEDIDAS@@</t>
         </is>
       </c>
-      <c r="D77" s="275" t="n"/>
-      <c r="E77" s="279" t="n"/>
-    </row>
-    <row r="78" ht="19.5" customHeight="1">
-      <c r="B78" s="18" t="inlineStr">
+      <c r="D80" s="275" t="n"/>
+      <c r="E80" s="279" t="n"/>
+    </row>
+    <row r="81" ht="19.5" customHeight="1">
+      <c r="B81" s="18" t="inlineStr">
         <is>
           <t>Plan de emergencia</t>
         </is>
       </c>
-      <c r="C78" s="168" t="inlineStr">
+      <c r="C81" s="168" t="inlineStr">
         <is>
           <t>@@RIESGOS_PLAN_EMERG@@</t>
         </is>
       </c>
-      <c r="D78" s="276" t="n"/>
-      <c r="E78" s="301" t="n"/>
-    </row>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81" ht="18.75" customHeight="1">
-      <c r="B81" s="58" t="n"/>
-      <c r="C81" s="67" t="inlineStr">
+      <c r="D81" s="276" t="n"/>
+      <c r="E81" s="301" t="n"/>
+    </row>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84" ht="18.75" customHeight="1">
+      <c r="B84" s="58" t="n"/>
+      <c r="C84" s="67" t="inlineStr">
         <is>
           <t>Día</t>
         </is>
       </c>
-      <c r="D81" s="67" t="inlineStr">
+      <c r="D84" s="67" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="E81" s="67" t="inlineStr">
+      <c r="E84" s="67" t="inlineStr">
         <is>
           <t>Año</t>
         </is>
       </c>
-      <c r="F81" s="51" t="n"/>
-      <c r="G81" s="51" t="n"/>
-      <c r="H81" s="51" t="n"/>
-      <c r="I81" s="51" t="n"/>
-      <c r="J81" s="51" t="n"/>
-      <c r="K81" s="51" t="n"/>
-    </row>
-    <row r="82" ht="18.75" customHeight="1">
-      <c r="B82" s="52" t="inlineStr">
-        <is>
-          <t>FECHA ELABORACIÓN:</t>
-        </is>
-      </c>
-      <c r="C82" s="57" t="inlineStr">
-        <is>
-          <t>@@ELAB_DIA@@</t>
-        </is>
-      </c>
-      <c r="D82" s="57" t="inlineStr">
-        <is>
-          <t>@@ELAB_MES@@</t>
-        </is>
-      </c>
-      <c r="E82" s="53" t="inlineStr">
-        <is>
-          <t>@@ELAB_ANIO@@</t>
-        </is>
-      </c>
-      <c r="F82" s="50" t="n"/>
-      <c r="G82" s="51" t="n"/>
-      <c r="H82" s="51" t="n"/>
-      <c r="I82" s="51" t="n"/>
-      <c r="J82" s="51" t="n"/>
-      <c r="K82" s="51" t="n"/>
-    </row>
-    <row r="83" ht="18.75" customHeight="1">
-      <c r="B83" s="52" t="inlineStr">
-        <is>
-          <t>ELABORADO POR:</t>
-        </is>
-      </c>
-      <c r="C83" s="302" t="inlineStr">
-        <is>
-          <t>@@ELABORADO_POR@@</t>
-        </is>
-      </c>
-      <c r="D83" s="275" t="n"/>
-      <c r="E83" s="270" t="n"/>
-      <c r="F83" s="173" t="inlineStr">
-        <is>
-          <t>FIRMA (JEFE PROYECTO)</t>
-        </is>
-      </c>
-      <c r="H83" s="51" t="n"/>
-      <c r="I83" s="51" t="n"/>
-      <c r="J83" s="51" t="n"/>
-      <c r="K83" s="51" t="n"/>
-    </row>
-    <row r="84" ht="18.75" customHeight="1">
-      <c r="B84" s="55" t="n"/>
-      <c r="C84" s="54" t="n"/>
-      <c r="D84" s="54" t="n"/>
-      <c r="E84" s="54" t="n"/>
       <c r="F84" s="51" t="n"/>
       <c r="G84" s="51" t="n"/>
       <c r="H84" s="51" t="n"/>
@@ -4988,36 +5039,62 @@
       <c r="J84" s="51" t="n"/>
       <c r="K84" s="51" t="n"/>
     </row>
-    <row r="85" ht="18.75" customHeight="1"/>
+    <row r="85" ht="18.75" customHeight="1">
+      <c r="B85" s="52" t="inlineStr">
+        <is>
+          <t>FECHA ELABORACIÓN:</t>
+        </is>
+      </c>
+      <c r="C85" s="57" t="inlineStr">
+        <is>
+          <t>@@ELAB_DIA@@</t>
+        </is>
+      </c>
+      <c r="D85" s="57" t="inlineStr">
+        <is>
+          <t>@@ELAB_MES@@</t>
+        </is>
+      </c>
+      <c r="E85" s="53" t="inlineStr">
+        <is>
+          <t>@@ELAB_ANIO@@</t>
+        </is>
+      </c>
+      <c r="F85" s="50" t="n"/>
+      <c r="G85" s="51" t="n"/>
+      <c r="H85" s="51" t="n"/>
+      <c r="I85" s="51" t="n"/>
+      <c r="J85" s="51" t="n"/>
+      <c r="K85" s="51" t="n"/>
+    </row>
     <row r="86" ht="18.75" customHeight="1">
-      <c r="B86" s="55" t="n"/>
-      <c r="C86" s="174" t="n"/>
-      <c r="D86" s="174" t="n"/>
-      <c r="E86" s="174" t="n"/>
-      <c r="F86" s="51" t="n"/>
-      <c r="G86" s="51" t="n"/>
+      <c r="B86" s="52" t="inlineStr">
+        <is>
+          <t>ELABORADO POR:</t>
+        </is>
+      </c>
+      <c r="C86" s="302" t="inlineStr">
+        <is>
+          <t>@@ELABORADO_POR@@</t>
+        </is>
+      </c>
+      <c r="D86" s="275" t="n"/>
+      <c r="E86" s="270" t="n"/>
+      <c r="F86" s="173" t="inlineStr">
+        <is>
+          <t>FIRMA (JEFE PROYECTO)</t>
+        </is>
+      </c>
       <c r="H86" s="51" t="n"/>
       <c r="I86" s="51" t="n"/>
       <c r="J86" s="51" t="n"/>
       <c r="K86" s="51" t="n"/>
     </row>
     <row r="87" ht="18.75" customHeight="1">
-      <c r="B87" s="58" t="n"/>
-      <c r="C87" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_DIA@@</t>
-        </is>
-      </c>
-      <c r="D87" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_MES@@</t>
-        </is>
-      </c>
-      <c r="E87" s="67" t="inlineStr">
-        <is>
-          <t>@@REV_ANIO@@</t>
-        </is>
-      </c>
+      <c r="B87" s="55" t="n"/>
+      <c r="C87" s="54" t="n"/>
+      <c r="D87" s="54" t="n"/>
+      <c r="E87" s="54" t="n"/>
       <c r="F87" s="51" t="n"/>
       <c r="G87" s="51" t="n"/>
       <c r="H87" s="51" t="n"/>
@@ -5025,162 +5102,196 @@
       <c r="J87" s="51" t="n"/>
       <c r="K87" s="51" t="n"/>
     </row>
-    <row r="88" ht="18.75" customHeight="1">
-      <c r="B88" s="52" t="inlineStr">
-        <is>
-          <t>FECHA REVISIÓN:</t>
-        </is>
-      </c>
-      <c r="C88" s="57" t="n"/>
-      <c r="D88" s="57" t="n"/>
-      <c r="E88" s="53" t="n"/>
-      <c r="F88" s="51" t="n"/>
-      <c r="G88" s="51" t="n"/>
-      <c r="H88" s="51" t="n"/>
-      <c r="I88" s="51" t="n"/>
-      <c r="J88" s="51" t="n"/>
-      <c r="K88" s="51" t="n"/>
-    </row>
+    <row r="88" ht="18.75" customHeight="1"/>
     <row r="89" ht="18.75" customHeight="1">
-      <c r="B89" s="52" t="inlineStr">
-        <is>
-          <t>REVISADO  POR:</t>
-        </is>
-      </c>
-      <c r="C89" s="302" t="inlineStr">
-        <is>
-          <t>@@REVISADO_POR@@</t>
-        </is>
-      </c>
-      <c r="D89" s="275" t="n"/>
-      <c r="E89" s="270" t="n"/>
-      <c r="F89" s="173" t="inlineStr">
-        <is>
-          <t>FIRMA (JEFE DEPARTAMENTO)</t>
-        </is>
-      </c>
+      <c r="B89" s="55" t="n"/>
+      <c r="C89" s="174" t="n"/>
+      <c r="D89" s="174" t="n"/>
+      <c r="E89" s="174" t="n"/>
+      <c r="F89" s="51" t="n"/>
+      <c r="G89" s="51" t="n"/>
       <c r="H89" s="51" t="n"/>
       <c r="I89" s="51" t="n"/>
       <c r="J89" s="51" t="n"/>
       <c r="K89" s="51" t="n"/>
     </row>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
+    <row r="90" ht="18.75" customHeight="1">
+      <c r="B90" s="58" t="n"/>
+      <c r="C90" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_DIA@@</t>
+        </is>
+      </c>
+      <c r="D90" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_MES@@</t>
+        </is>
+      </c>
+      <c r="E90" s="67" t="inlineStr">
+        <is>
+          <t>@@REV_ANIO@@</t>
+        </is>
+      </c>
+      <c r="F90" s="51" t="n"/>
+      <c r="G90" s="51" t="n"/>
+      <c r="H90" s="51" t="n"/>
+      <c r="I90" s="51" t="n"/>
+      <c r="J90" s="51" t="n"/>
+      <c r="K90" s="51" t="n"/>
+    </row>
+    <row r="91" ht="18.75" customHeight="1">
+      <c r="B91" s="52" t="inlineStr">
+        <is>
+          <t>FECHA REVISIÓN:</t>
+        </is>
+      </c>
+      <c r="C91" s="57" t="n"/>
+      <c r="D91" s="57" t="n"/>
+      <c r="E91" s="53" t="n"/>
+      <c r="F91" s="51" t="n"/>
+      <c r="G91" s="51" t="n"/>
+      <c r="H91" s="51" t="n"/>
+      <c r="I91" s="51" t="n"/>
+      <c r="J91" s="51" t="n"/>
+      <c r="K91" s="51" t="n"/>
+    </row>
+    <row r="92" ht="18.75" customHeight="1">
+      <c r="B92" s="52" t="inlineStr">
+        <is>
+          <t>REVISADO  POR:</t>
+        </is>
+      </c>
+      <c r="C92" s="302" t="inlineStr">
+        <is>
+          <t>@@REVISADO_POR@@</t>
+        </is>
+      </c>
+      <c r="D92" s="275" t="n"/>
+      <c r="E92" s="270" t="n"/>
+      <c r="F92" s="173" t="inlineStr">
+        <is>
+          <t>FIRMA (JEFE DEPARTAMENTO)</t>
+        </is>
+      </c>
+      <c r="H92" s="51" t="n"/>
+      <c r="I92" s="51" t="n"/>
+      <c r="J92" s="51" t="n"/>
+      <c r="K92" s="51" t="n"/>
+    </row>
     <row r="93"/>
-    <row r="94" ht="18.75" customHeight="1">
-      <c r="B94" s="169" t="inlineStr">
-        <is>
-          <t>@@NOTA_PERMISO_CIRCULACION@@</t>
-        </is>
-      </c>
-    </row>
+    <row r="94"/>
     <row r="95"/>
     <row r="96"/>
-    <row r="97"/>
+    <row r="97" ht="18.75" customHeight="1">
+      <c r="B97" s="169" t="inlineStr">
+        <is>
+          <t>@@NOTA_PERMISO_CIRCULACION@@</t>
+        </is>
+      </c>
+    </row>
     <row r="98"/>
     <row r="99"/>
     <row r="100"/>
   </sheetData>
   <mergeCells count="98">
+    <mergeCell ref="C9:S10"/>
     <mergeCell ref="Q21:R21"/>
-    <mergeCell ref="C9:S10"/>
     <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C80:E80"/>
     <mergeCell ref="C30:P30"/>
     <mergeCell ref="F68:P68"/>
-    <mergeCell ref="B94:K94"/>
+    <mergeCell ref="F86:G86"/>
     <mergeCell ref="C41:D41"/>
-    <mergeCell ref="B15:B16"/>
     <mergeCell ref="F70:P70"/>
-    <mergeCell ref="C43:D43"/>
     <mergeCell ref="G42:P42"/>
     <mergeCell ref="D15:D16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C43:D43"/>
     <mergeCell ref="G8:J8"/>
+    <mergeCell ref="F72:P72"/>
     <mergeCell ref="L25:P25"/>
-    <mergeCell ref="F72:P72"/>
     <mergeCell ref="E58:P58"/>
-    <mergeCell ref="C77:E77"/>
     <mergeCell ref="C23:P23"/>
     <mergeCell ref="E50:P50"/>
-    <mergeCell ref="B37:B44"/>
     <mergeCell ref="F71:P71"/>
-    <mergeCell ref="G37:P37"/>
+    <mergeCell ref="Q17:R17"/>
     <mergeCell ref="C4:S5"/>
-    <mergeCell ref="Q17:R17"/>
     <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B78:E78"/>
     <mergeCell ref="E52:P52"/>
     <mergeCell ref="J15:L15"/>
     <mergeCell ref="D27:F27"/>
-    <mergeCell ref="F63:P63"/>
-    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="C45:D45"/>
     <mergeCell ref="E59:P59"/>
     <mergeCell ref="G41:P41"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E46:P46"/>
-    <mergeCell ref="L24:P24"/>
+    <mergeCell ref="C47:D47"/>
     <mergeCell ref="C29:P29"/>
     <mergeCell ref="H27:J27"/>
+    <mergeCell ref="L24:P24"/>
+    <mergeCell ref="E61:P61"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="G43:P43"/>
     <mergeCell ref="E40:F40"/>
     <mergeCell ref="D25:F25"/>
     <mergeCell ref="L8:P8"/>
     <mergeCell ref="E57:P57"/>
+    <mergeCell ref="C81:E81"/>
     <mergeCell ref="E54:P54"/>
-    <mergeCell ref="B47:B60"/>
-    <mergeCell ref="F62:P62"/>
-    <mergeCell ref="E47:P47"/>
+    <mergeCell ref="F75:P75"/>
     <mergeCell ref="E56:P56"/>
-    <mergeCell ref="C89:E89"/>
     <mergeCell ref="B7:S7"/>
+    <mergeCell ref="C79:E79"/>
     <mergeCell ref="M15:S15"/>
-    <mergeCell ref="F64:P64"/>
+    <mergeCell ref="F73:P73"/>
+    <mergeCell ref="G45:P45"/>
     <mergeCell ref="E60:P60"/>
-    <mergeCell ref="F89:G89"/>
-    <mergeCell ref="E39:F39"/>
+    <mergeCell ref="G47:P47"/>
     <mergeCell ref="E44:F44"/>
     <mergeCell ref="G44:P44"/>
+    <mergeCell ref="F74:P74"/>
+    <mergeCell ref="G46:P46"/>
     <mergeCell ref="G40:P40"/>
     <mergeCell ref="Q20:R20"/>
     <mergeCell ref="E15:E16"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="G15:G16"/>
+    <mergeCell ref="B50:B63"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="H24:J24"/>
+    <mergeCell ref="C46:D46"/>
     <mergeCell ref="F66:P66"/>
-    <mergeCell ref="C78:E78"/>
-    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="C92:E92"/>
+    <mergeCell ref="E62:P62"/>
+    <mergeCell ref="F92:G92"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="L27:P27"/>
-    <mergeCell ref="E51:P51"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="F15:F16"/>
     <mergeCell ref="D28:P28"/>
     <mergeCell ref="E43:F43"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="E51:P51"/>
     <mergeCell ref="F69:P69"/>
+    <mergeCell ref="E63:P63"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="E42:F42"/>
     <mergeCell ref="F65:P65"/>
     <mergeCell ref="C12:S13"/>
     <mergeCell ref="Q18:R18"/>
-    <mergeCell ref="C76:E76"/>
-    <mergeCell ref="B75:E75"/>
+    <mergeCell ref="B97:K97"/>
     <mergeCell ref="E49:P49"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="Q19:R19"/>
     <mergeCell ref="D24:F24"/>
-    <mergeCell ref="G39:P39"/>
+    <mergeCell ref="E45:F45"/>
     <mergeCell ref="E53:P53"/>
-    <mergeCell ref="C83:E83"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="G38:P38"/>
+    <mergeCell ref="C86:E86"/>
     <mergeCell ref="F67:P67"/>
     <mergeCell ref="E55:P55"/>
-    <mergeCell ref="C37:D37"/>
+    <mergeCell ref="B40:B47"/>
     <mergeCell ref="C15:C16"/>
-    <mergeCell ref="E37:F37"/>
-    <mergeCell ref="E48:P48"/>
     <mergeCell ref="H25:J25"/>
+    <mergeCell ref="E47:F47"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="C8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list">

</xml_diff>

<commit_message>
Viático: tarifas actualizadas (profesional 86.921 / 40% 34.768; administrativo 59.320 / 40% 23.728); SW v17.
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/plantilla_ficha_terreno.xlsx
+++ b/assets/plantilla_ficha_terreno.xlsx
@@ -3625,10 +3625,10 @@
         </is>
       </c>
       <c r="O33" s="282" t="n">
-        <v>85721</v>
+        <v>86921</v>
       </c>
       <c r="P33" s="283" t="n">
-        <v>34288</v>
+        <v>34768</v>
       </c>
       <c r="Q33" s="10" t="n"/>
       <c r="R33" s="10" t="n"/>
@@ -3781,10 +3781,10 @@
         </is>
       </c>
       <c r="O37" s="284" t="n">
-        <v>58501</v>
+        <v>59320</v>
       </c>
       <c r="P37" s="285" t="n">
-        <v>23400</v>
+        <v>23728</v>
       </c>
       <c r="Q37" s="1" t="n"/>
       <c r="R37" s="1" t="n"/>
@@ -4959,7 +4959,6 @@
       <c r="O75" s="276" t="n"/>
       <c r="P75" s="271" t="n"/>
     </row>
-    <row r="76"/>
     <row r="77" ht="15.75" customHeight="1"/>
     <row r="78" ht="18.75" customHeight="1">
       <c r="B78" s="300" t="inlineStr">
@@ -5013,8 +5012,6 @@
       <c r="D81" s="276" t="n"/>
       <c r="E81" s="301" t="n"/>
     </row>
-    <row r="82"/>
-    <row r="83"/>
     <row r="84" ht="18.75" customHeight="1">
       <c r="B84" s="58" t="n"/>
       <c r="C84" s="67" t="inlineStr">
@@ -5178,10 +5175,6 @@
       <c r="J92" s="51" t="n"/>
       <c r="K92" s="51" t="n"/>
     </row>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97" ht="18.75" customHeight="1">
       <c r="B97" s="169" t="inlineStr">
         <is>
@@ -5189,9 +5182,6 @@
         </is>
       </c>
     </row>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
   </sheetData>
   <mergeCells count="98">
     <mergeCell ref="C9:S10"/>
@@ -5202,10 +5192,10 @@
     <mergeCell ref="F68:P68"/>
     <mergeCell ref="F86:G86"/>
     <mergeCell ref="C41:D41"/>
+    <mergeCell ref="B15:B16"/>
     <mergeCell ref="F70:P70"/>
     <mergeCell ref="G42:P42"/>
     <mergeCell ref="D15:D16"/>
-    <mergeCell ref="B15:B16"/>
     <mergeCell ref="C43:D43"/>
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="F72:P72"/>
@@ -5266,8 +5256,8 @@
     <mergeCell ref="F92:G92"/>
     <mergeCell ref="E41:F41"/>
     <mergeCell ref="L27:P27"/>
+    <mergeCell ref="F15:F16"/>
     <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="F15:F16"/>
     <mergeCell ref="D28:P28"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="E51:P51"/>

</xml_diff>